<commit_message>
Versión casa: finalizados los centralizadores SEC hasta 4to
</commit_message>
<xml_diff>
--- a/public/templates/cs56.xlsx
+++ b/public/templates/cs56.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\saat\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A7EED6E-DC6F-4E9C-960B-6E9EAE301014}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6657F06C-4BAC-4D09-BAB3-3718DF104736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1344,12 +1344,81 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="27" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="27" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="62" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="62" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="62" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1359,121 +1428,52 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="62" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="62" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="62" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="27" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="27" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1669,7 +1669,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>59</xdr:col>
-      <xdr:colOff>904875</xdr:colOff>
+      <xdr:colOff>706755</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
@@ -2063,443 +2063,444 @@
   <cols>
     <col min="1" max="1" width="2.5546875" customWidth="1"/>
     <col min="2" max="2" width="30.6640625" customWidth="1"/>
-    <col min="3" max="59" width="3.88671875" customWidth="1"/>
-    <col min="60" max="60" width="32.88671875" customWidth="1"/>
+    <col min="3" max="58" width="3.88671875" customWidth="1"/>
+    <col min="59" max="59" width="6.77734375" customWidth="1"/>
+    <col min="60" max="60" width="39" customWidth="1"/>
     <col min="61" max="72" width="4" customWidth="1"/>
     <col min="73" max="80" width="3.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:72" x14ac:dyDescent="0.3">
-      <c r="A2" s="110" t="s">
+      <c r="A2" s="113" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="110"/>
-      <c r="C2" s="110"/>
-      <c r="D2" s="110"/>
-      <c r="E2" s="110"/>
-      <c r="F2" s="110"/>
-      <c r="G2" s="110"/>
-      <c r="H2" s="110"/>
-      <c r="I2" s="110"/>
-      <c r="J2" s="110"/>
-      <c r="K2" s="110"/>
-      <c r="L2" s="110"/>
-      <c r="M2" s="110"/>
-      <c r="N2" s="110"/>
-      <c r="O2" s="110"/>
-      <c r="P2" s="110"/>
-      <c r="Q2" s="110"/>
-      <c r="R2" s="110"/>
-      <c r="S2" s="110"/>
-      <c r="T2" s="110"/>
-      <c r="U2" s="110"/>
-      <c r="V2" s="110"/>
-      <c r="W2" s="110"/>
-      <c r="X2" s="110"/>
-      <c r="Y2" s="110"/>
-      <c r="Z2" s="110"/>
-      <c r="AA2" s="110"/>
-      <c r="AB2" s="110"/>
-      <c r="AC2" s="110"/>
-      <c r="AD2" s="110"/>
-      <c r="AE2" s="110"/>
-      <c r="AF2" s="110"/>
-      <c r="AG2" s="110"/>
-      <c r="AH2" s="110"/>
-      <c r="AI2" s="110"/>
-      <c r="AJ2" s="110"/>
-      <c r="AK2" s="110"/>
-      <c r="AL2" s="110"/>
-      <c r="AM2" s="110"/>
-      <c r="AN2" s="110"/>
-      <c r="AO2" s="110"/>
-      <c r="AP2" s="110"/>
-      <c r="AQ2" s="110"/>
-      <c r="AR2" s="110"/>
-      <c r="AS2" s="110"/>
-      <c r="AT2" s="110"/>
-      <c r="AU2" s="110"/>
-      <c r="AV2" s="110"/>
-      <c r="AW2" s="110"/>
-      <c r="AX2" s="110"/>
-      <c r="AY2" s="110"/>
-      <c r="AZ2" s="110"/>
-      <c r="BA2" s="110"/>
-      <c r="BB2" s="110"/>
-      <c r="BC2" s="110"/>
-      <c r="BD2" s="110"/>
-      <c r="BE2" s="110"/>
-      <c r="BF2" s="110"/>
-      <c r="BG2" s="125" t="str">
+      <c r="B2" s="113"/>
+      <c r="C2" s="113"/>
+      <c r="D2" s="113"/>
+      <c r="E2" s="113"/>
+      <c r="F2" s="113"/>
+      <c r="G2" s="113"/>
+      <c r="H2" s="113"/>
+      <c r="I2" s="113"/>
+      <c r="J2" s="113"/>
+      <c r="K2" s="113"/>
+      <c r="L2" s="113"/>
+      <c r="M2" s="113"/>
+      <c r="N2" s="113"/>
+      <c r="O2" s="113"/>
+      <c r="P2" s="113"/>
+      <c r="Q2" s="113"/>
+      <c r="R2" s="113"/>
+      <c r="S2" s="113"/>
+      <c r="T2" s="113"/>
+      <c r="U2" s="113"/>
+      <c r="V2" s="113"/>
+      <c r="W2" s="113"/>
+      <c r="X2" s="113"/>
+      <c r="Y2" s="113"/>
+      <c r="Z2" s="113"/>
+      <c r="AA2" s="113"/>
+      <c r="AB2" s="113"/>
+      <c r="AC2" s="113"/>
+      <c r="AD2" s="113"/>
+      <c r="AE2" s="113"/>
+      <c r="AF2" s="113"/>
+      <c r="AG2" s="113"/>
+      <c r="AH2" s="113"/>
+      <c r="AI2" s="113"/>
+      <c r="AJ2" s="113"/>
+      <c r="AK2" s="113"/>
+      <c r="AL2" s="113"/>
+      <c r="AM2" s="113"/>
+      <c r="AN2" s="113"/>
+      <c r="AO2" s="113"/>
+      <c r="AP2" s="113"/>
+      <c r="AQ2" s="113"/>
+      <c r="AR2" s="113"/>
+      <c r="AS2" s="113"/>
+      <c r="AT2" s="113"/>
+      <c r="AU2" s="113"/>
+      <c r="AV2" s="113"/>
+      <c r="AW2" s="113"/>
+      <c r="AX2" s="113"/>
+      <c r="AY2" s="113"/>
+      <c r="AZ2" s="113"/>
+      <c r="BA2" s="113"/>
+      <c r="BB2" s="113"/>
+      <c r="BC2" s="113"/>
+      <c r="BD2" s="113"/>
+      <c r="BE2" s="113"/>
+      <c r="BF2" s="113"/>
+      <c r="BG2" s="133" t="str">
         <f>A2</f>
         <v>CUADRO GENERAL DE NOTAS</v>
       </c>
-      <c r="BH2" s="125"/>
-      <c r="BI2" s="125"/>
-      <c r="BJ2" s="125"/>
-      <c r="BK2" s="125"/>
-      <c r="BL2" s="125"/>
-      <c r="BM2" s="125"/>
-      <c r="BN2" s="125"/>
-      <c r="BO2" s="125"/>
-      <c r="BP2" s="125"/>
-      <c r="BQ2" s="125"/>
-      <c r="BR2" s="125"/>
-      <c r="BS2" s="125"/>
-      <c r="BT2" s="125"/>
+      <c r="BH2" s="133"/>
+      <c r="BI2" s="133"/>
+      <c r="BJ2" s="133"/>
+      <c r="BK2" s="133"/>
+      <c r="BL2" s="133"/>
+      <c r="BM2" s="133"/>
+      <c r="BN2" s="133"/>
+      <c r="BO2" s="133"/>
+      <c r="BP2" s="133"/>
+      <c r="BQ2" s="133"/>
+      <c r="BR2" s="133"/>
+      <c r="BS2" s="133"/>
+      <c r="BT2" s="133"/>
     </row>
     <row r="3" spans="1:72" x14ac:dyDescent="0.3">
-      <c r="A3" s="111" t="s">
+      <c r="A3" s="114" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="111"/>
-      <c r="C3" s="111"/>
-      <c r="D3" s="111"/>
-      <c r="E3" s="111"/>
-      <c r="F3" s="111"/>
-      <c r="G3" s="111"/>
-      <c r="H3" s="111"/>
-      <c r="I3" s="111"/>
-      <c r="J3" s="111"/>
-      <c r="K3" s="111"/>
-      <c r="L3" s="111"/>
-      <c r="M3" s="111"/>
-      <c r="N3" s="111"/>
-      <c r="O3" s="111"/>
-      <c r="P3" s="111"/>
-      <c r="Q3" s="111"/>
-      <c r="R3" s="111"/>
-      <c r="S3" s="111"/>
-      <c r="T3" s="111"/>
-      <c r="U3" s="111"/>
-      <c r="V3" s="111"/>
-      <c r="W3" s="111"/>
-      <c r="X3" s="111"/>
-      <c r="Y3" s="111"/>
-      <c r="Z3" s="111"/>
-      <c r="AA3" s="111"/>
-      <c r="AB3" s="111"/>
-      <c r="AC3" s="111"/>
-      <c r="AD3" s="111"/>
-      <c r="AE3" s="111"/>
-      <c r="AF3" s="111"/>
-      <c r="AG3" s="111"/>
-      <c r="AH3" s="111"/>
-      <c r="AI3" s="111"/>
-      <c r="AJ3" s="111"/>
-      <c r="AK3" s="111"/>
-      <c r="AL3" s="111"/>
-      <c r="AM3" s="111"/>
-      <c r="AN3" s="111"/>
-      <c r="AO3" s="111"/>
-      <c r="AP3" s="111"/>
-      <c r="AQ3" s="111"/>
-      <c r="AR3" s="111"/>
-      <c r="AS3" s="111"/>
-      <c r="AT3" s="111"/>
-      <c r="AU3" s="111"/>
-      <c r="AV3" s="111"/>
-      <c r="AW3" s="111"/>
-      <c r="AX3" s="111"/>
-      <c r="AY3" s="111"/>
-      <c r="AZ3" s="111"/>
-      <c r="BA3" s="111"/>
-      <c r="BB3" s="111"/>
-      <c r="BC3" s="111"/>
-      <c r="BD3" s="111"/>
-      <c r="BE3" s="111"/>
-      <c r="BF3" s="111"/>
-      <c r="BG3" s="130" t="str">
+      <c r="B3" s="114"/>
+      <c r="C3" s="114"/>
+      <c r="D3" s="114"/>
+      <c r="E3" s="114"/>
+      <c r="F3" s="114"/>
+      <c r="G3" s="114"/>
+      <c r="H3" s="114"/>
+      <c r="I3" s="114"/>
+      <c r="J3" s="114"/>
+      <c r="K3" s="114"/>
+      <c r="L3" s="114"/>
+      <c r="M3" s="114"/>
+      <c r="N3" s="114"/>
+      <c r="O3" s="114"/>
+      <c r="P3" s="114"/>
+      <c r="Q3" s="114"/>
+      <c r="R3" s="114"/>
+      <c r="S3" s="114"/>
+      <c r="T3" s="114"/>
+      <c r="U3" s="114"/>
+      <c r="V3" s="114"/>
+      <c r="W3" s="114"/>
+      <c r="X3" s="114"/>
+      <c r="Y3" s="114"/>
+      <c r="Z3" s="114"/>
+      <c r="AA3" s="114"/>
+      <c r="AB3" s="114"/>
+      <c r="AC3" s="114"/>
+      <c r="AD3" s="114"/>
+      <c r="AE3" s="114"/>
+      <c r="AF3" s="114"/>
+      <c r="AG3" s="114"/>
+      <c r="AH3" s="114"/>
+      <c r="AI3" s="114"/>
+      <c r="AJ3" s="114"/>
+      <c r="AK3" s="114"/>
+      <c r="AL3" s="114"/>
+      <c r="AM3" s="114"/>
+      <c r="AN3" s="114"/>
+      <c r="AO3" s="114"/>
+      <c r="AP3" s="114"/>
+      <c r="AQ3" s="114"/>
+      <c r="AR3" s="114"/>
+      <c r="AS3" s="114"/>
+      <c r="AT3" s="114"/>
+      <c r="AU3" s="114"/>
+      <c r="AV3" s="114"/>
+      <c r="AW3" s="114"/>
+      <c r="AX3" s="114"/>
+      <c r="AY3" s="114"/>
+      <c r="AZ3" s="114"/>
+      <c r="BA3" s="114"/>
+      <c r="BB3" s="114"/>
+      <c r="BC3" s="114"/>
+      <c r="BD3" s="114"/>
+      <c r="BE3" s="114"/>
+      <c r="BF3" s="114"/>
+      <c r="BG3" s="96" t="str">
         <f t="shared" ref="BG3:BG5" si="0">A3</f>
         <v>(CONSEJEROS Y DIRECCIONES TÉCNICAS)</v>
       </c>
-      <c r="BH3" s="130"/>
-      <c r="BI3" s="130"/>
-      <c r="BJ3" s="130"/>
-      <c r="BK3" s="130"/>
-      <c r="BL3" s="130"/>
-      <c r="BM3" s="130"/>
-      <c r="BN3" s="130"/>
-      <c r="BO3" s="130"/>
-      <c r="BP3" s="130"/>
-      <c r="BQ3" s="130"/>
-      <c r="BR3" s="130"/>
-      <c r="BS3" s="130"/>
-      <c r="BT3" s="130"/>
+      <c r="BH3" s="96"/>
+      <c r="BI3" s="96"/>
+      <c r="BJ3" s="96"/>
+      <c r="BK3" s="96"/>
+      <c r="BL3" s="96"/>
+      <c r="BM3" s="96"/>
+      <c r="BN3" s="96"/>
+      <c r="BO3" s="96"/>
+      <c r="BP3" s="96"/>
+      <c r="BQ3" s="96"/>
+      <c r="BR3" s="96"/>
+      <c r="BS3" s="96"/>
+      <c r="BT3" s="96"/>
     </row>
     <row r="4" spans="1:72" x14ac:dyDescent="0.3">
-      <c r="A4" s="112"/>
-      <c r="B4" s="112"/>
-      <c r="C4" s="112"/>
-      <c r="D4" s="112"/>
-      <c r="E4" s="112"/>
-      <c r="F4" s="112"/>
-      <c r="G4" s="112"/>
-      <c r="H4" s="112"/>
-      <c r="I4" s="112"/>
-      <c r="J4" s="112"/>
-      <c r="K4" s="112"/>
-      <c r="L4" s="112"/>
-      <c r="M4" s="112"/>
-      <c r="N4" s="112"/>
-      <c r="O4" s="112"/>
-      <c r="P4" s="112"/>
-      <c r="Q4" s="112"/>
-      <c r="R4" s="112"/>
-      <c r="S4" s="112"/>
-      <c r="T4" s="112"/>
-      <c r="U4" s="112"/>
-      <c r="V4" s="112"/>
-      <c r="W4" s="112"/>
-      <c r="X4" s="112"/>
-      <c r="Y4" s="112"/>
-      <c r="Z4" s="112"/>
-      <c r="AA4" s="112"/>
-      <c r="AB4" s="112"/>
-      <c r="AC4" s="112"/>
-      <c r="AD4" s="112"/>
-      <c r="AE4" s="112"/>
-      <c r="AF4" s="112"/>
-      <c r="AG4" s="112"/>
-      <c r="AH4" s="112"/>
-      <c r="AI4" s="112"/>
-      <c r="AJ4" s="112"/>
-      <c r="AK4" s="112"/>
-      <c r="AL4" s="112"/>
-      <c r="AM4" s="112"/>
-      <c r="AN4" s="112"/>
-      <c r="AO4" s="112"/>
-      <c r="AP4" s="112"/>
-      <c r="AQ4" s="112"/>
-      <c r="AR4" s="112"/>
-      <c r="AS4" s="112"/>
-      <c r="AT4" s="112"/>
-      <c r="AU4" s="112"/>
-      <c r="AV4" s="112"/>
-      <c r="AW4" s="112"/>
-      <c r="AX4" s="112"/>
-      <c r="AY4" s="112"/>
-      <c r="AZ4" s="112"/>
-      <c r="BA4" s="112"/>
-      <c r="BB4" s="112"/>
-      <c r="BC4" s="112"/>
-      <c r="BD4" s="112"/>
-      <c r="BE4" s="112"/>
-      <c r="BF4" s="112"/>
-      <c r="BG4" s="129">
+      <c r="A4" s="115"/>
+      <c r="B4" s="115"/>
+      <c r="C4" s="115"/>
+      <c r="D4" s="115"/>
+      <c r="E4" s="115"/>
+      <c r="F4" s="115"/>
+      <c r="G4" s="115"/>
+      <c r="H4" s="115"/>
+      <c r="I4" s="115"/>
+      <c r="J4" s="115"/>
+      <c r="K4" s="115"/>
+      <c r="L4" s="115"/>
+      <c r="M4" s="115"/>
+      <c r="N4" s="115"/>
+      <c r="O4" s="115"/>
+      <c r="P4" s="115"/>
+      <c r="Q4" s="115"/>
+      <c r="R4" s="115"/>
+      <c r="S4" s="115"/>
+      <c r="T4" s="115"/>
+      <c r="U4" s="115"/>
+      <c r="V4" s="115"/>
+      <c r="W4" s="115"/>
+      <c r="X4" s="115"/>
+      <c r="Y4" s="115"/>
+      <c r="Z4" s="115"/>
+      <c r="AA4" s="115"/>
+      <c r="AB4" s="115"/>
+      <c r="AC4" s="115"/>
+      <c r="AD4" s="115"/>
+      <c r="AE4" s="115"/>
+      <c r="AF4" s="115"/>
+      <c r="AG4" s="115"/>
+      <c r="AH4" s="115"/>
+      <c r="AI4" s="115"/>
+      <c r="AJ4" s="115"/>
+      <c r="AK4" s="115"/>
+      <c r="AL4" s="115"/>
+      <c r="AM4" s="115"/>
+      <c r="AN4" s="115"/>
+      <c r="AO4" s="115"/>
+      <c r="AP4" s="115"/>
+      <c r="AQ4" s="115"/>
+      <c r="AR4" s="115"/>
+      <c r="AS4" s="115"/>
+      <c r="AT4" s="115"/>
+      <c r="AU4" s="115"/>
+      <c r="AV4" s="115"/>
+      <c r="AW4" s="115"/>
+      <c r="AX4" s="115"/>
+      <c r="AY4" s="115"/>
+      <c r="AZ4" s="115"/>
+      <c r="BA4" s="115"/>
+      <c r="BB4" s="115"/>
+      <c r="BC4" s="115"/>
+      <c r="BD4" s="115"/>
+      <c r="BE4" s="115"/>
+      <c r="BF4" s="115"/>
+      <c r="BG4" s="95">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="BH4" s="129"/>
-      <c r="BI4" s="129"/>
-      <c r="BJ4" s="129"/>
-      <c r="BK4" s="129"/>
-      <c r="BL4" s="129"/>
-      <c r="BM4" s="129"/>
-      <c r="BN4" s="129"/>
-      <c r="BO4" s="129"/>
-      <c r="BP4" s="129"/>
-      <c r="BQ4" s="129"/>
-      <c r="BR4" s="129"/>
-      <c r="BS4" s="129"/>
-      <c r="BT4" s="129"/>
+      <c r="BH4" s="95"/>
+      <c r="BI4" s="95"/>
+      <c r="BJ4" s="95"/>
+      <c r="BK4" s="95"/>
+      <c r="BL4" s="95"/>
+      <c r="BM4" s="95"/>
+      <c r="BN4" s="95"/>
+      <c r="BO4" s="95"/>
+      <c r="BP4" s="95"/>
+      <c r="BQ4" s="95"/>
+      <c r="BR4" s="95"/>
+      <c r="BS4" s="95"/>
+      <c r="BT4" s="95"/>
     </row>
     <row r="5" spans="1:72" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="113"/>
-      <c r="B5" s="113"/>
-      <c r="C5" s="113"/>
-      <c r="D5" s="113"/>
-      <c r="E5" s="113"/>
-      <c r="F5" s="113"/>
-      <c r="G5" s="113"/>
-      <c r="H5" s="113"/>
-      <c r="I5" s="113"/>
-      <c r="J5" s="113"/>
-      <c r="K5" s="113"/>
-      <c r="L5" s="113"/>
-      <c r="M5" s="113"/>
-      <c r="N5" s="113"/>
-      <c r="O5" s="113"/>
-      <c r="P5" s="113"/>
-      <c r="Q5" s="113"/>
-      <c r="R5" s="113"/>
-      <c r="S5" s="113"/>
-      <c r="T5" s="113"/>
-      <c r="U5" s="113"/>
-      <c r="V5" s="113"/>
-      <c r="W5" s="113"/>
-      <c r="X5" s="113"/>
-      <c r="Y5" s="113"/>
-      <c r="Z5" s="113"/>
-      <c r="AA5" s="113"/>
-      <c r="AB5" s="113"/>
-      <c r="AC5" s="113"/>
-      <c r="AD5" s="113"/>
-      <c r="AE5" s="113"/>
-      <c r="AF5" s="113"/>
-      <c r="AG5" s="113"/>
-      <c r="AH5" s="113"/>
-      <c r="AI5" s="113"/>
-      <c r="AJ5" s="113"/>
-      <c r="AK5" s="113"/>
-      <c r="AL5" s="113"/>
-      <c r="AM5" s="113"/>
-      <c r="AN5" s="113"/>
-      <c r="AO5" s="113"/>
-      <c r="AP5" s="113"/>
-      <c r="AQ5" s="113"/>
-      <c r="AR5" s="113"/>
-      <c r="AS5" s="113"/>
-      <c r="AT5" s="113"/>
-      <c r="AU5" s="113"/>
-      <c r="AV5" s="113"/>
-      <c r="AW5" s="113"/>
-      <c r="AX5" s="113"/>
-      <c r="AY5" s="113"/>
-      <c r="AZ5" s="113"/>
-      <c r="BA5" s="113"/>
-      <c r="BB5" s="113"/>
-      <c r="BC5" s="113"/>
-      <c r="BD5" s="113"/>
-      <c r="BE5" s="113"/>
-      <c r="BF5" s="113"/>
-      <c r="BG5" s="128">
+      <c r="A5" s="116"/>
+      <c r="B5" s="116"/>
+      <c r="C5" s="116"/>
+      <c r="D5" s="116"/>
+      <c r="E5" s="116"/>
+      <c r="F5" s="116"/>
+      <c r="G5" s="116"/>
+      <c r="H5" s="116"/>
+      <c r="I5" s="116"/>
+      <c r="J5" s="116"/>
+      <c r="K5" s="116"/>
+      <c r="L5" s="116"/>
+      <c r="M5" s="116"/>
+      <c r="N5" s="116"/>
+      <c r="O5" s="116"/>
+      <c r="P5" s="116"/>
+      <c r="Q5" s="116"/>
+      <c r="R5" s="116"/>
+      <c r="S5" s="116"/>
+      <c r="T5" s="116"/>
+      <c r="U5" s="116"/>
+      <c r="V5" s="116"/>
+      <c r="W5" s="116"/>
+      <c r="X5" s="116"/>
+      <c r="Y5" s="116"/>
+      <c r="Z5" s="116"/>
+      <c r="AA5" s="116"/>
+      <c r="AB5" s="116"/>
+      <c r="AC5" s="116"/>
+      <c r="AD5" s="116"/>
+      <c r="AE5" s="116"/>
+      <c r="AF5" s="116"/>
+      <c r="AG5" s="116"/>
+      <c r="AH5" s="116"/>
+      <c r="AI5" s="116"/>
+      <c r="AJ5" s="116"/>
+      <c r="AK5" s="116"/>
+      <c r="AL5" s="116"/>
+      <c r="AM5" s="116"/>
+      <c r="AN5" s="116"/>
+      <c r="AO5" s="116"/>
+      <c r="AP5" s="116"/>
+      <c r="AQ5" s="116"/>
+      <c r="AR5" s="116"/>
+      <c r="AS5" s="116"/>
+      <c r="AT5" s="116"/>
+      <c r="AU5" s="116"/>
+      <c r="AV5" s="116"/>
+      <c r="AW5" s="116"/>
+      <c r="AX5" s="116"/>
+      <c r="AY5" s="116"/>
+      <c r="AZ5" s="116"/>
+      <c r="BA5" s="116"/>
+      <c r="BB5" s="116"/>
+      <c r="BC5" s="116"/>
+      <c r="BD5" s="116"/>
+      <c r="BE5" s="116"/>
+      <c r="BF5" s="116"/>
+      <c r="BG5" s="94">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="BH5" s="128"/>
-      <c r="BI5" s="128"/>
-      <c r="BJ5" s="128"/>
-      <c r="BK5" s="128"/>
-      <c r="BL5" s="128"/>
-      <c r="BM5" s="128"/>
-      <c r="BN5" s="128"/>
-      <c r="BO5" s="128"/>
-      <c r="BP5" s="128"/>
-      <c r="BQ5" s="128"/>
-      <c r="BR5" s="128"/>
-      <c r="BS5" s="128"/>
-      <c r="BT5" s="128"/>
+      <c r="BH5" s="94"/>
+      <c r="BI5" s="94"/>
+      <c r="BJ5" s="94"/>
+      <c r="BK5" s="94"/>
+      <c r="BL5" s="94"/>
+      <c r="BM5" s="94"/>
+      <c r="BN5" s="94"/>
+      <c r="BO5" s="94"/>
+      <c r="BP5" s="94"/>
+      <c r="BQ5" s="94"/>
+      <c r="BR5" s="94"/>
+      <c r="BS5" s="94"/>
+      <c r="BT5" s="94"/>
     </row>
     <row r="6" spans="1:72" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="104" t="s">
+      <c r="A6" s="107" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="108" t="s">
+      <c r="B6" s="109" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="101" t="s">
+      <c r="C6" s="100" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="102"/>
-      <c r="E6" s="102"/>
-      <c r="F6" s="103"/>
-      <c r="G6" s="101" t="s">
+      <c r="D6" s="101"/>
+      <c r="E6" s="101"/>
+      <c r="F6" s="102"/>
+      <c r="G6" s="100" t="s">
         <v>20</v>
       </c>
-      <c r="H6" s="102"/>
-      <c r="I6" s="102"/>
-      <c r="J6" s="103"/>
-      <c r="K6" s="121" t="s">
+      <c r="H6" s="101"/>
+      <c r="I6" s="101"/>
+      <c r="J6" s="102"/>
+      <c r="K6" s="129" t="s">
         <v>30</v>
       </c>
-      <c r="L6" s="122"/>
-      <c r="M6" s="123"/>
-      <c r="N6" s="124"/>
-      <c r="O6" s="101" t="s">
+      <c r="L6" s="130"/>
+      <c r="M6" s="131"/>
+      <c r="N6" s="132"/>
+      <c r="O6" s="100" t="s">
         <v>19</v>
       </c>
-      <c r="P6" s="102"/>
-      <c r="Q6" s="102"/>
-      <c r="R6" s="103"/>
-      <c r="S6" s="97" t="s">
+      <c r="P6" s="101"/>
+      <c r="Q6" s="101"/>
+      <c r="R6" s="102"/>
+      <c r="S6" s="124" t="s">
         <v>2</v>
       </c>
-      <c r="T6" s="94"/>
-      <c r="U6" s="95"/>
-      <c r="V6" s="98"/>
-      <c r="W6" s="97" t="s">
+      <c r="T6" s="117"/>
+      <c r="U6" s="118"/>
+      <c r="V6" s="125"/>
+      <c r="W6" s="124" t="s">
         <v>16</v>
       </c>
-      <c r="X6" s="94"/>
-      <c r="Y6" s="95"/>
-      <c r="Z6" s="98"/>
-      <c r="AA6" s="94" t="s">
+      <c r="X6" s="117"/>
+      <c r="Y6" s="118"/>
+      <c r="Z6" s="125"/>
+      <c r="AA6" s="117" t="s">
         <v>3</v>
       </c>
-      <c r="AB6" s="94"/>
-      <c r="AC6" s="95"/>
-      <c r="AD6" s="96"/>
-      <c r="AE6" s="97" t="s">
+      <c r="AB6" s="117"/>
+      <c r="AC6" s="118"/>
+      <c r="AD6" s="119"/>
+      <c r="AE6" s="124" t="s">
         <v>26</v>
       </c>
-      <c r="AF6" s="94"/>
-      <c r="AG6" s="95"/>
-      <c r="AH6" s="98"/>
-      <c r="AI6" s="118" t="s">
+      <c r="AF6" s="117"/>
+      <c r="AG6" s="118"/>
+      <c r="AH6" s="125"/>
+      <c r="AI6" s="126" t="s">
         <v>31</v>
       </c>
-      <c r="AJ6" s="119"/>
-      <c r="AK6" s="119"/>
-      <c r="AL6" s="120"/>
-      <c r="AM6" s="97" t="s">
+      <c r="AJ6" s="127"/>
+      <c r="AK6" s="127"/>
+      <c r="AL6" s="128"/>
+      <c r="AM6" s="124" t="s">
         <v>17</v>
       </c>
-      <c r="AN6" s="94"/>
-      <c r="AO6" s="95"/>
-      <c r="AP6" s="98"/>
-      <c r="AQ6" s="97" t="s">
+      <c r="AN6" s="117"/>
+      <c r="AO6" s="118"/>
+      <c r="AP6" s="125"/>
+      <c r="AQ6" s="124" t="s">
         <v>18</v>
       </c>
-      <c r="AR6" s="94"/>
-      <c r="AS6" s="95"/>
-      <c r="AT6" s="98"/>
-      <c r="AU6" s="101" t="s">
+      <c r="AR6" s="117"/>
+      <c r="AS6" s="118"/>
+      <c r="AT6" s="125"/>
+      <c r="AU6" s="100" t="s">
         <v>21</v>
       </c>
-      <c r="AV6" s="102"/>
-      <c r="AW6" s="102"/>
-      <c r="AX6" s="103"/>
-      <c r="AY6" s="94" t="s">
+      <c r="AV6" s="101"/>
+      <c r="AW6" s="101"/>
+      <c r="AX6" s="102"/>
+      <c r="AY6" s="117" t="s">
         <v>4</v>
       </c>
-      <c r="AZ6" s="94"/>
-      <c r="BA6" s="95"/>
-      <c r="BB6" s="96"/>
-      <c r="BC6" s="114" t="s">
+      <c r="AZ6" s="117"/>
+      <c r="BA6" s="118"/>
+      <c r="BB6" s="119"/>
+      <c r="BC6" s="120" t="s">
         <v>5</v>
       </c>
-      <c r="BD6" s="115"/>
-      <c r="BE6" s="116"/>
-      <c r="BF6" s="117"/>
-      <c r="BG6" s="104" t="s">
+      <c r="BD6" s="121"/>
+      <c r="BE6" s="122"/>
+      <c r="BF6" s="123"/>
+      <c r="BG6" s="107" t="s">
         <v>0</v>
       </c>
-      <c r="BH6" s="108" t="s">
+      <c r="BH6" s="109" t="s">
         <v>1</v>
       </c>
-      <c r="BI6" s="131" t="s">
+      <c r="BI6" s="97" t="s">
         <v>15</v>
       </c>
-      <c r="BJ6" s="132"/>
-      <c r="BK6" s="132"/>
-      <c r="BL6" s="132"/>
-      <c r="BM6" s="131" t="s">
+      <c r="BJ6" s="98"/>
+      <c r="BK6" s="98"/>
+      <c r="BL6" s="98"/>
+      <c r="BM6" s="97" t="s">
         <v>8</v>
       </c>
-      <c r="BN6" s="132"/>
-      <c r="BO6" s="132"/>
-      <c r="BP6" s="133"/>
-      <c r="BQ6" s="101" t="s">
+      <c r="BN6" s="98"/>
+      <c r="BO6" s="98"/>
+      <c r="BP6" s="99"/>
+      <c r="BQ6" s="100" t="s">
         <v>20</v>
       </c>
-      <c r="BR6" s="102"/>
-      <c r="BS6" s="102"/>
-      <c r="BT6" s="103"/>
+      <c r="BR6" s="101"/>
+      <c r="BS6" s="101"/>
+      <c r="BT6" s="102"/>
     </row>
     <row r="7" spans="1:72" x14ac:dyDescent="0.3">
-      <c r="A7" s="105"/>
-      <c r="B7" s="109"/>
+      <c r="A7" s="108"/>
+      <c r="B7" s="110"/>
       <c r="C7" s="2" t="s">
         <v>27</v>
       </c>
@@ -2668,8 +2669,8 @@
       <c r="BF7" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="BG7" s="105"/>
-      <c r="BH7" s="109"/>
+      <c r="BG7" s="108"/>
+      <c r="BH7" s="110"/>
       <c r="BI7" s="11" t="s">
         <v>27</v>
       </c>
@@ -6938,10 +6939,10 @@
       </c>
     </row>
     <row r="38" spans="1:72" x14ac:dyDescent="0.3">
-      <c r="A38" s="106" t="s">
+      <c r="A38" s="111" t="s">
         <v>9</v>
       </c>
-      <c r="B38" s="107"/>
+      <c r="B38" s="112"/>
       <c r="C38" s="62" t="str">
         <f t="shared" ref="C38:F38" si="23">IF(SUM(C8:C37)=0,"",AVERAGE(C8:C37))</f>
         <v/>
@@ -7166,10 +7167,10 @@
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="BG38" s="106" t="s">
+      <c r="BG38" s="111" t="s">
         <v>9</v>
       </c>
-      <c r="BH38" s="107"/>
+      <c r="BH38" s="112"/>
       <c r="BI38" s="73" t="str">
         <f t="shared" ref="BI38:BT38" si="27">IF(SUM(BI8:BI37)=0,"",AVERAGE(BI8:BI37))</f>
         <v/>
@@ -7220,10 +7221,10 @@
       </c>
     </row>
     <row r="39" spans="1:72" x14ac:dyDescent="0.3">
-      <c r="A39" s="92" t="s">
+      <c r="A39" s="103" t="s">
         <v>10</v>
       </c>
-      <c r="B39" s="93"/>
+      <c r="B39" s="104"/>
       <c r="C39" s="62" t="str">
         <f t="shared" ref="C39:F39" si="28">IF(SUM(C8:C37)=0,"",MEDIAN(C8:C37))</f>
         <v/>
@@ -7448,10 +7449,10 @@
         <f t="shared" si="31"/>
         <v/>
       </c>
-      <c r="BG39" s="92" t="s">
+      <c r="BG39" s="103" t="s">
         <v>10</v>
       </c>
-      <c r="BH39" s="93"/>
+      <c r="BH39" s="104"/>
       <c r="BI39" s="73" t="str">
         <f t="shared" ref="BI39:BT39" si="32">IF(SUM(BI8:BI37)=0,"",MEDIAN(BI8:BI37))</f>
         <v/>
@@ -7502,10 +7503,10 @@
       </c>
     </row>
     <row r="40" spans="1:72" x14ac:dyDescent="0.3">
-      <c r="A40" s="92" t="s">
+      <c r="A40" s="103" t="s">
         <v>11</v>
       </c>
-      <c r="B40" s="93"/>
+      <c r="B40" s="104"/>
       <c r="C40" s="62" t="str">
         <f t="shared" ref="C40:F40" si="33">IF(SUM(C8:C37)=0,"",MAX(C8:C37))</f>
         <v/>
@@ -7730,10 +7731,10 @@
         <f t="shared" si="36"/>
         <v/>
       </c>
-      <c r="BG40" s="92" t="s">
+      <c r="BG40" s="103" t="s">
         <v>11</v>
       </c>
-      <c r="BH40" s="93"/>
+      <c r="BH40" s="104"/>
       <c r="BI40" s="73" t="str">
         <f t="shared" ref="BI40:BT40" si="37">IF(SUM(BI8:BI37)=0,"",MAX(BI8:BI37))</f>
         <v/>
@@ -7784,10 +7785,10 @@
       </c>
     </row>
     <row r="41" spans="1:72" x14ac:dyDescent="0.3">
-      <c r="A41" s="92" t="s">
+      <c r="A41" s="103" t="s">
         <v>12</v>
       </c>
-      <c r="B41" s="93"/>
+      <c r="B41" s="104"/>
       <c r="C41" s="62" t="str">
         <f t="shared" ref="C41:F41" si="38">IF(SUM(C8:C37)=0,"",MIN(C8:C37))</f>
         <v/>
@@ -8012,10 +8013,10 @@
         <f t="shared" si="41"/>
         <v/>
       </c>
-      <c r="BG41" s="92" t="s">
+      <c r="BG41" s="103" t="s">
         <v>12</v>
       </c>
-      <c r="BH41" s="93"/>
+      <c r="BH41" s="104"/>
       <c r="BI41" s="73" t="str">
         <f t="shared" ref="BI41:BT41" si="42">IF(SUM(BI8:BI37)=0,"",MIN(BI8:BI37))</f>
         <v/>
@@ -8066,10 +8067,10 @@
       </c>
     </row>
     <row r="42" spans="1:72" x14ac:dyDescent="0.3">
-      <c r="A42" s="99" t="s">
+      <c r="A42" s="134" t="s">
         <v>13</v>
       </c>
-      <c r="B42" s="100"/>
+      <c r="B42" s="135"/>
       <c r="C42" s="77" t="str">
         <f t="shared" ref="C42:F42" si="43">IF(C38="","",COUNTIF(C8:C37,"&lt;51")/COUNT(C8:C37)*100)</f>
         <v/>
@@ -8294,10 +8295,10 @@
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="BG42" s="134" t="s">
+      <c r="BG42" s="105" t="s">
         <v>13</v>
       </c>
-      <c r="BH42" s="135"/>
+      <c r="BH42" s="106"/>
       <c r="BI42" s="88" t="str">
         <f t="shared" ref="BI42:BT42" si="47">IF(BI38="","",COUNTIF(BI8:BI37,"&lt;51")/COUNT(BI8:BI37)*100)</f>
         <v/>
@@ -8355,80 +8356,80 @@
     <row r="49" spans="2:77" ht="12.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="50" spans="2:77" ht="12.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="51" spans="2:77" x14ac:dyDescent="0.3">
-      <c r="B51" s="126" t="s">
+      <c r="B51" s="92" t="s">
         <v>22</v>
       </c>
-      <c r="C51" s="126"/>
-      <c r="D51" s="126"/>
-      <c r="E51" s="126"/>
-      <c r="F51" s="126"/>
-      <c r="G51" s="126"/>
-      <c r="H51" s="126"/>
-      <c r="I51" s="126"/>
-      <c r="J51" s="126"/>
+      <c r="C51" s="92"/>
+      <c r="D51" s="92"/>
+      <c r="E51" s="92"/>
+      <c r="F51" s="92"/>
+      <c r="G51" s="92"/>
+      <c r="H51" s="92"/>
+      <c r="I51" s="92"/>
+      <c r="J51" s="92"/>
       <c r="K51" s="1"/>
       <c r="L51" s="1"/>
       <c r="M51" s="1"/>
       <c r="N51" s="1"/>
       <c r="O51" s="1"/>
       <c r="P51" s="1"/>
-      <c r="Q51" s="126" t="s">
+      <c r="Q51" s="92" t="s">
         <v>22</v>
       </c>
-      <c r="R51" s="126"/>
-      <c r="S51" s="126"/>
-      <c r="T51" s="126"/>
-      <c r="U51" s="126"/>
-      <c r="V51" s="126"/>
-      <c r="W51" s="126"/>
-      <c r="X51" s="126"/>
-      <c r="Y51" s="126"/>
-      <c r="Z51" s="126"/>
-      <c r="AA51" s="126"/>
-      <c r="AB51" s="126"/>
-      <c r="AC51" s="126"/>
+      <c r="R51" s="92"/>
+      <c r="S51" s="92"/>
+      <c r="T51" s="92"/>
+      <c r="U51" s="92"/>
+      <c r="V51" s="92"/>
+      <c r="W51" s="92"/>
+      <c r="X51" s="92"/>
+      <c r="Y51" s="92"/>
+      <c r="Z51" s="92"/>
+      <c r="AA51" s="92"/>
+      <c r="AB51" s="92"/>
+      <c r="AC51" s="92"/>
       <c r="AD51" s="1"/>
       <c r="AE51" s="1"/>
       <c r="AF51" s="1"/>
       <c r="AG51" s="1"/>
-      <c r="AH51" s="126" t="s">
+      <c r="AH51" s="92" t="s">
         <v>22</v>
       </c>
-      <c r="AI51" s="126"/>
-      <c r="AJ51" s="126"/>
-      <c r="AK51" s="126"/>
-      <c r="AL51" s="126"/>
-      <c r="AM51" s="126"/>
-      <c r="AN51" s="126"/>
-      <c r="AO51" s="126"/>
-      <c r="AP51" s="126"/>
-      <c r="AQ51" s="126"/>
-      <c r="AR51" s="126"/>
-      <c r="AS51" s="126"/>
+      <c r="AI51" s="92"/>
+      <c r="AJ51" s="92"/>
+      <c r="AK51" s="92"/>
+      <c r="AL51" s="92"/>
+      <c r="AM51" s="92"/>
+      <c r="AN51" s="92"/>
+      <c r="AO51" s="92"/>
+      <c r="AP51" s="92"/>
+      <c r="AQ51" s="92"/>
+      <c r="AR51" s="92"/>
+      <c r="AS51" s="92"/>
       <c r="AT51" s="1"/>
       <c r="AU51" s="1"/>
       <c r="AV51" s="1"/>
       <c r="AW51" s="1"/>
       <c r="AX51" s="1"/>
       <c r="AY51" s="1"/>
-      <c r="BG51" s="126" t="s">
+      <c r="BG51" s="92" t="s">
         <v>22</v>
       </c>
-      <c r="BH51" s="126"/>
+      <c r="BH51" s="92"/>
       <c r="BI51" s="90"/>
       <c r="BJ51" s="76"/>
       <c r="BK51" s="76"/>
-      <c r="BL51" s="126" t="s">
+      <c r="BL51" s="92" t="s">
         <v>22</v>
       </c>
-      <c r="BM51" s="126"/>
-      <c r="BN51" s="126"/>
-      <c r="BO51" s="126"/>
-      <c r="BP51" s="126"/>
-      <c r="BQ51" s="126"/>
-      <c r="BR51" s="126"/>
-      <c r="BS51" s="126"/>
-      <c r="BT51" s="126"/>
+      <c r="BM51" s="92"/>
+      <c r="BN51" s="92"/>
+      <c r="BO51" s="92"/>
+      <c r="BP51" s="92"/>
+      <c r="BQ51" s="92"/>
+      <c r="BR51" s="92"/>
+      <c r="BS51" s="92"/>
+      <c r="BT51" s="92"/>
       <c r="BU51" s="76"/>
       <c r="BV51" s="76"/>
       <c r="BW51" s="76"/>
@@ -8436,56 +8437,56 @@
       <c r="BY51" s="76"/>
     </row>
     <row r="52" spans="2:77" x14ac:dyDescent="0.3">
-      <c r="B52" s="127" t="s">
+      <c r="B52" s="93" t="s">
         <v>23</v>
       </c>
-      <c r="C52" s="127"/>
-      <c r="D52" s="127"/>
-      <c r="E52" s="127"/>
-      <c r="F52" s="127"/>
-      <c r="G52" s="127"/>
-      <c r="H52" s="127"/>
-      <c r="I52" s="127"/>
-      <c r="J52" s="127"/>
+      <c r="C52" s="93"/>
+      <c r="D52" s="93"/>
+      <c r="E52" s="93"/>
+      <c r="F52" s="93"/>
+      <c r="G52" s="93"/>
+      <c r="H52" s="93"/>
+      <c r="I52" s="93"/>
+      <c r="J52" s="93"/>
       <c r="K52" s="1"/>
       <c r="L52" s="1"/>
       <c r="M52" s="1"/>
       <c r="N52" s="1"/>
       <c r="O52" s="1"/>
       <c r="P52" s="1"/>
-      <c r="Q52" s="127" t="s">
+      <c r="Q52" s="93" t="s">
         <v>24</v>
       </c>
-      <c r="R52" s="127"/>
-      <c r="S52" s="127"/>
-      <c r="T52" s="127"/>
-      <c r="U52" s="127"/>
-      <c r="V52" s="127"/>
-      <c r="W52" s="127"/>
-      <c r="X52" s="127"/>
-      <c r="Y52" s="127"/>
-      <c r="Z52" s="127"/>
-      <c r="AA52" s="127"/>
-      <c r="AB52" s="127"/>
-      <c r="AC52" s="127"/>
+      <c r="R52" s="93"/>
+      <c r="S52" s="93"/>
+      <c r="T52" s="93"/>
+      <c r="U52" s="93"/>
+      <c r="V52" s="93"/>
+      <c r="W52" s="93"/>
+      <c r="X52" s="93"/>
+      <c r="Y52" s="93"/>
+      <c r="Z52" s="93"/>
+      <c r="AA52" s="93"/>
+      <c r="AB52" s="93"/>
+      <c r="AC52" s="93"/>
       <c r="AD52" s="1"/>
       <c r="AE52" s="1"/>
       <c r="AF52" s="1"/>
       <c r="AG52" s="1"/>
-      <c r="AH52" s="127" t="s">
+      <c r="AH52" s="93" t="s">
         <v>25</v>
       </c>
-      <c r="AI52" s="127"/>
-      <c r="AJ52" s="127"/>
-      <c r="AK52" s="127"/>
-      <c r="AL52" s="127"/>
-      <c r="AM52" s="127"/>
-      <c r="AN52" s="127"/>
-      <c r="AO52" s="127"/>
-      <c r="AP52" s="127"/>
-      <c r="AQ52" s="127"/>
-      <c r="AR52" s="127"/>
-      <c r="AS52" s="127"/>
+      <c r="AI52" s="93"/>
+      <c r="AJ52" s="93"/>
+      <c r="AK52" s="93"/>
+      <c r="AL52" s="93"/>
+      <c r="AM52" s="93"/>
+      <c r="AN52" s="93"/>
+      <c r="AO52" s="93"/>
+      <c r="AP52" s="93"/>
+      <c r="AQ52" s="93"/>
+      <c r="AR52" s="93"/>
+      <c r="AS52" s="93"/>
       <c r="AT52" s="1"/>
       <c r="AU52" s="1"/>
       <c r="AV52" s="1"/>
@@ -8495,24 +8496,24 @@
       <c r="BE52" t="s">
         <v>38</v>
       </c>
-      <c r="BG52" s="127" t="s">
+      <c r="BG52" s="93" t="s">
         <v>23</v>
       </c>
-      <c r="BH52" s="127"/>
+      <c r="BH52" s="93"/>
       <c r="BI52" s="91"/>
       <c r="BJ52" s="76"/>
       <c r="BK52" s="76"/>
-      <c r="BL52" s="127" t="s">
+      <c r="BL52" s="93" t="s">
         <v>25</v>
       </c>
-      <c r="BM52" s="127"/>
-      <c r="BN52" s="127"/>
-      <c r="BO52" s="127"/>
-      <c r="BP52" s="127"/>
-      <c r="BQ52" s="127"/>
-      <c r="BR52" s="127"/>
-      <c r="BS52" s="127"/>
-      <c r="BT52" s="127"/>
+      <c r="BM52" s="93"/>
+      <c r="BN52" s="93"/>
+      <c r="BO52" s="93"/>
+      <c r="BP52" s="93"/>
+      <c r="BQ52" s="93"/>
+      <c r="BR52" s="93"/>
+      <c r="BS52" s="93"/>
+      <c r="BT52" s="93"/>
       <c r="BU52" s="76"/>
       <c r="BV52" s="76"/>
       <c r="BW52" s="76"/>
@@ -8523,29 +8524,19 @@
     </row>
   </sheetData>
   <mergeCells count="49">
-    <mergeCell ref="BL51:BT51"/>
-    <mergeCell ref="BG52:BH52"/>
-    <mergeCell ref="BL52:BT52"/>
-    <mergeCell ref="B51:J51"/>
-    <mergeCell ref="B52:J52"/>
-    <mergeCell ref="BG5:BT5"/>
-    <mergeCell ref="BG4:BT4"/>
-    <mergeCell ref="BG3:BT3"/>
-    <mergeCell ref="BI6:BL6"/>
-    <mergeCell ref="BM6:BP6"/>
-    <mergeCell ref="BQ6:BT6"/>
-    <mergeCell ref="Q51:AC51"/>
-    <mergeCell ref="Q52:AC52"/>
-    <mergeCell ref="AH51:AS51"/>
-    <mergeCell ref="AH52:AS52"/>
-    <mergeCell ref="BG41:BH41"/>
-    <mergeCell ref="BG42:BH42"/>
-    <mergeCell ref="BG51:BH51"/>
-    <mergeCell ref="BG6:BG7"/>
-    <mergeCell ref="BH6:BH7"/>
-    <mergeCell ref="BG38:BH38"/>
-    <mergeCell ref="BG39:BH39"/>
-    <mergeCell ref="BG40:BH40"/>
+    <mergeCell ref="BG2:BT2"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="AA6:AD6"/>
+    <mergeCell ref="AE6:AH6"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="G6:J6"/>
+    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="W6:Z6"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="B6:B7"/>
     <mergeCell ref="A2:BF2"/>
     <mergeCell ref="A3:BF3"/>
     <mergeCell ref="A4:BF4"/>
@@ -8559,19 +8550,29 @@
     <mergeCell ref="AM6:AP6"/>
     <mergeCell ref="AQ6:AT6"/>
     <mergeCell ref="K6:N6"/>
-    <mergeCell ref="BG2:BT2"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="AA6:AD6"/>
-    <mergeCell ref="AE6:AH6"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="G6:J6"/>
-    <mergeCell ref="C6:F6"/>
-    <mergeCell ref="W6:Z6"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="BG41:BH41"/>
+    <mergeCell ref="BG42:BH42"/>
+    <mergeCell ref="BG51:BH51"/>
+    <mergeCell ref="BG6:BG7"/>
+    <mergeCell ref="BH6:BH7"/>
+    <mergeCell ref="BG38:BH38"/>
+    <mergeCell ref="BG39:BH39"/>
+    <mergeCell ref="BG40:BH40"/>
+    <mergeCell ref="BG5:BT5"/>
+    <mergeCell ref="BG4:BT4"/>
+    <mergeCell ref="BG3:BT3"/>
+    <mergeCell ref="BI6:BL6"/>
+    <mergeCell ref="BM6:BP6"/>
+    <mergeCell ref="BQ6:BT6"/>
+    <mergeCell ref="BL51:BT51"/>
+    <mergeCell ref="BG52:BH52"/>
+    <mergeCell ref="BL52:BT52"/>
+    <mergeCell ref="B51:J51"/>
+    <mergeCell ref="B52:J52"/>
+    <mergeCell ref="Q51:AC51"/>
+    <mergeCell ref="Q52:AC52"/>
+    <mergeCell ref="AH51:AS51"/>
+    <mergeCell ref="AH52:AS52"/>
   </mergeCells>
   <conditionalFormatting sqref="C8:BF37 BI8:BT37">
     <cfRule type="cellIs" dxfId="1" priority="3" operator="between">
@@ -8584,7 +8585,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.21249999999999999" right="0.25" top="0.46643518518518517" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="10000" scale="64" fitToWidth="2" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="10000" scale="63" fitToWidth="2" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <colBreaks count="1" manualBreakCount="1">
     <brk id="58" max="1048575" man="1"/>
   </colBreaks>

</xml_diff>

<commit_message>
GENERACION DE CENTRALIZADORES HASTA 6TO SEC
</commit_message>
<xml_diff>
--- a/public/templates/cs56.xlsx
+++ b/public/templates/cs56.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\saat\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6657F06C-4BAC-4D09-BAB3-3718DF104736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B7F7ADF-F82C-47C7-BF44-82E3F99D90C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Central" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Central!$A$1:$CD$52</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -34,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="39">
   <si>
     <t>Nº</t>
   </si>
@@ -151,7 +154,7 @@
     <t>1 de 2</t>
   </si>
   <si>
-    <t>1 de 1</t>
+    <t>2 de 2</t>
   </si>
 </sst>
 </file>
@@ -1079,7 +1082,7 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="136">
+  <cellXfs count="137">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1295,9 +1298,6 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="1" fontId="25" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1344,138 +1344,142 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="62" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="62" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="62" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="27" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="27" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="27" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="27" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="62" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="62" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="62" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="71">
     <cellStyle name="20% - Accent1" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -2058,448 +2062,448 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:BY52"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A2:CD52"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.5546875" customWidth="1"/>
-    <col min="2" max="2" width="30.6640625" customWidth="1"/>
-    <col min="3" max="58" width="3.88671875" customWidth="1"/>
-    <col min="59" max="59" width="6.77734375" customWidth="1"/>
+    <col min="1" max="1" width="2.5703125" customWidth="1"/>
+    <col min="2" max="2" width="30.7109375" customWidth="1"/>
+    <col min="3" max="58" width="3.85546875" customWidth="1"/>
+    <col min="59" max="59" width="6.7109375" customWidth="1"/>
     <col min="60" max="60" width="39" customWidth="1"/>
-    <col min="61" max="72" width="4" customWidth="1"/>
-    <col min="73" max="80" width="3.5546875" customWidth="1"/>
+    <col min="61" max="72" width="5.5703125" customWidth="1"/>
+    <col min="73" max="80" width="3.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:72" x14ac:dyDescent="0.3">
-      <c r="A2" s="113" t="s">
+    <row r="2" spans="1:72" x14ac:dyDescent="0.25">
+      <c r="A2" s="111" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="113"/>
-      <c r="C2" s="113"/>
-      <c r="D2" s="113"/>
-      <c r="E2" s="113"/>
-      <c r="F2" s="113"/>
-      <c r="G2" s="113"/>
-      <c r="H2" s="113"/>
-      <c r="I2" s="113"/>
-      <c r="J2" s="113"/>
-      <c r="K2" s="113"/>
-      <c r="L2" s="113"/>
-      <c r="M2" s="113"/>
-      <c r="N2" s="113"/>
-      <c r="O2" s="113"/>
-      <c r="P2" s="113"/>
-      <c r="Q2" s="113"/>
-      <c r="R2" s="113"/>
-      <c r="S2" s="113"/>
-      <c r="T2" s="113"/>
-      <c r="U2" s="113"/>
-      <c r="V2" s="113"/>
-      <c r="W2" s="113"/>
-      <c r="X2" s="113"/>
-      <c r="Y2" s="113"/>
-      <c r="Z2" s="113"/>
-      <c r="AA2" s="113"/>
-      <c r="AB2" s="113"/>
-      <c r="AC2" s="113"/>
-      <c r="AD2" s="113"/>
-      <c r="AE2" s="113"/>
-      <c r="AF2" s="113"/>
-      <c r="AG2" s="113"/>
-      <c r="AH2" s="113"/>
-      <c r="AI2" s="113"/>
-      <c r="AJ2" s="113"/>
-      <c r="AK2" s="113"/>
-      <c r="AL2" s="113"/>
-      <c r="AM2" s="113"/>
-      <c r="AN2" s="113"/>
-      <c r="AO2" s="113"/>
-      <c r="AP2" s="113"/>
-      <c r="AQ2" s="113"/>
-      <c r="AR2" s="113"/>
-      <c r="AS2" s="113"/>
-      <c r="AT2" s="113"/>
-      <c r="AU2" s="113"/>
-      <c r="AV2" s="113"/>
-      <c r="AW2" s="113"/>
-      <c r="AX2" s="113"/>
-      <c r="AY2" s="113"/>
-      <c r="AZ2" s="113"/>
-      <c r="BA2" s="113"/>
-      <c r="BB2" s="113"/>
-      <c r="BC2" s="113"/>
-      <c r="BD2" s="113"/>
-      <c r="BE2" s="113"/>
-      <c r="BF2" s="113"/>
-      <c r="BG2" s="133" t="str">
+      <c r="B2" s="111"/>
+      <c r="C2" s="111"/>
+      <c r="D2" s="111"/>
+      <c r="E2" s="111"/>
+      <c r="F2" s="111"/>
+      <c r="G2" s="111"/>
+      <c r="H2" s="111"/>
+      <c r="I2" s="111"/>
+      <c r="J2" s="111"/>
+      <c r="K2" s="111"/>
+      <c r="L2" s="111"/>
+      <c r="M2" s="111"/>
+      <c r="N2" s="111"/>
+      <c r="O2" s="111"/>
+      <c r="P2" s="111"/>
+      <c r="Q2" s="111"/>
+      <c r="R2" s="111"/>
+      <c r="S2" s="111"/>
+      <c r="T2" s="111"/>
+      <c r="U2" s="111"/>
+      <c r="V2" s="111"/>
+      <c r="W2" s="111"/>
+      <c r="X2" s="111"/>
+      <c r="Y2" s="111"/>
+      <c r="Z2" s="111"/>
+      <c r="AA2" s="111"/>
+      <c r="AB2" s="111"/>
+      <c r="AC2" s="111"/>
+      <c r="AD2" s="111"/>
+      <c r="AE2" s="111"/>
+      <c r="AF2" s="111"/>
+      <c r="AG2" s="111"/>
+      <c r="AH2" s="111"/>
+      <c r="AI2" s="111"/>
+      <c r="AJ2" s="111"/>
+      <c r="AK2" s="111"/>
+      <c r="AL2" s="111"/>
+      <c r="AM2" s="111"/>
+      <c r="AN2" s="111"/>
+      <c r="AO2" s="111"/>
+      <c r="AP2" s="111"/>
+      <c r="AQ2" s="111"/>
+      <c r="AR2" s="111"/>
+      <c r="AS2" s="111"/>
+      <c r="AT2" s="111"/>
+      <c r="AU2" s="111"/>
+      <c r="AV2" s="111"/>
+      <c r="AW2" s="111"/>
+      <c r="AX2" s="111"/>
+      <c r="AY2" s="111"/>
+      <c r="AZ2" s="111"/>
+      <c r="BA2" s="111"/>
+      <c r="BB2" s="111"/>
+      <c r="BC2" s="111"/>
+      <c r="BD2" s="111"/>
+      <c r="BE2" s="111"/>
+      <c r="BF2" s="111"/>
+      <c r="BG2" s="92" t="str">
         <f>A2</f>
         <v>CUADRO GENERAL DE NOTAS</v>
       </c>
-      <c r="BH2" s="133"/>
-      <c r="BI2" s="133"/>
-      <c r="BJ2" s="133"/>
-      <c r="BK2" s="133"/>
-      <c r="BL2" s="133"/>
-      <c r="BM2" s="133"/>
-      <c r="BN2" s="133"/>
-      <c r="BO2" s="133"/>
-      <c r="BP2" s="133"/>
-      <c r="BQ2" s="133"/>
-      <c r="BR2" s="133"/>
-      <c r="BS2" s="133"/>
-      <c r="BT2" s="133"/>
+      <c r="BH2" s="92"/>
+      <c r="BI2" s="92"/>
+      <c r="BJ2" s="92"/>
+      <c r="BK2" s="92"/>
+      <c r="BL2" s="92"/>
+      <c r="BM2" s="92"/>
+      <c r="BN2" s="92"/>
+      <c r="BO2" s="92"/>
+      <c r="BP2" s="92"/>
+      <c r="BQ2" s="92"/>
+      <c r="BR2" s="92"/>
+      <c r="BS2" s="92"/>
+      <c r="BT2" s="92"/>
     </row>
-    <row r="3" spans="1:72" x14ac:dyDescent="0.3">
-      <c r="A3" s="114" t="s">
+    <row r="3" spans="1:72" x14ac:dyDescent="0.25">
+      <c r="A3" s="112" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="114"/>
-      <c r="C3" s="114"/>
-      <c r="D3" s="114"/>
-      <c r="E3" s="114"/>
-      <c r="F3" s="114"/>
-      <c r="G3" s="114"/>
-      <c r="H3" s="114"/>
-      <c r="I3" s="114"/>
-      <c r="J3" s="114"/>
-      <c r="K3" s="114"/>
-      <c r="L3" s="114"/>
-      <c r="M3" s="114"/>
-      <c r="N3" s="114"/>
-      <c r="O3" s="114"/>
-      <c r="P3" s="114"/>
-      <c r="Q3" s="114"/>
-      <c r="R3" s="114"/>
-      <c r="S3" s="114"/>
-      <c r="T3" s="114"/>
-      <c r="U3" s="114"/>
-      <c r="V3" s="114"/>
-      <c r="W3" s="114"/>
-      <c r="X3" s="114"/>
-      <c r="Y3" s="114"/>
-      <c r="Z3" s="114"/>
-      <c r="AA3" s="114"/>
-      <c r="AB3" s="114"/>
-      <c r="AC3" s="114"/>
-      <c r="AD3" s="114"/>
-      <c r="AE3" s="114"/>
-      <c r="AF3" s="114"/>
-      <c r="AG3" s="114"/>
-      <c r="AH3" s="114"/>
-      <c r="AI3" s="114"/>
-      <c r="AJ3" s="114"/>
-      <c r="AK3" s="114"/>
-      <c r="AL3" s="114"/>
-      <c r="AM3" s="114"/>
-      <c r="AN3" s="114"/>
-      <c r="AO3" s="114"/>
-      <c r="AP3" s="114"/>
-      <c r="AQ3" s="114"/>
-      <c r="AR3" s="114"/>
-      <c r="AS3" s="114"/>
-      <c r="AT3" s="114"/>
-      <c r="AU3" s="114"/>
-      <c r="AV3" s="114"/>
-      <c r="AW3" s="114"/>
-      <c r="AX3" s="114"/>
-      <c r="AY3" s="114"/>
-      <c r="AZ3" s="114"/>
-      <c r="BA3" s="114"/>
-      <c r="BB3" s="114"/>
-      <c r="BC3" s="114"/>
-      <c r="BD3" s="114"/>
-      <c r="BE3" s="114"/>
-      <c r="BF3" s="114"/>
-      <c r="BG3" s="96" t="str">
+      <c r="B3" s="112"/>
+      <c r="C3" s="112"/>
+      <c r="D3" s="112"/>
+      <c r="E3" s="112"/>
+      <c r="F3" s="112"/>
+      <c r="G3" s="112"/>
+      <c r="H3" s="112"/>
+      <c r="I3" s="112"/>
+      <c r="J3" s="112"/>
+      <c r="K3" s="112"/>
+      <c r="L3" s="112"/>
+      <c r="M3" s="112"/>
+      <c r="N3" s="112"/>
+      <c r="O3" s="112"/>
+      <c r="P3" s="112"/>
+      <c r="Q3" s="112"/>
+      <c r="R3" s="112"/>
+      <c r="S3" s="112"/>
+      <c r="T3" s="112"/>
+      <c r="U3" s="112"/>
+      <c r="V3" s="112"/>
+      <c r="W3" s="112"/>
+      <c r="X3" s="112"/>
+      <c r="Y3" s="112"/>
+      <c r="Z3" s="112"/>
+      <c r="AA3" s="112"/>
+      <c r="AB3" s="112"/>
+      <c r="AC3" s="112"/>
+      <c r="AD3" s="112"/>
+      <c r="AE3" s="112"/>
+      <c r="AF3" s="112"/>
+      <c r="AG3" s="112"/>
+      <c r="AH3" s="112"/>
+      <c r="AI3" s="112"/>
+      <c r="AJ3" s="112"/>
+      <c r="AK3" s="112"/>
+      <c r="AL3" s="112"/>
+      <c r="AM3" s="112"/>
+      <c r="AN3" s="112"/>
+      <c r="AO3" s="112"/>
+      <c r="AP3" s="112"/>
+      <c r="AQ3" s="112"/>
+      <c r="AR3" s="112"/>
+      <c r="AS3" s="112"/>
+      <c r="AT3" s="112"/>
+      <c r="AU3" s="112"/>
+      <c r="AV3" s="112"/>
+      <c r="AW3" s="112"/>
+      <c r="AX3" s="112"/>
+      <c r="AY3" s="112"/>
+      <c r="AZ3" s="112"/>
+      <c r="BA3" s="112"/>
+      <c r="BB3" s="112"/>
+      <c r="BC3" s="112"/>
+      <c r="BD3" s="112"/>
+      <c r="BE3" s="112"/>
+      <c r="BF3" s="112"/>
+      <c r="BG3" s="131" t="str">
         <f t="shared" ref="BG3:BG5" si="0">A3</f>
         <v>(CONSEJEROS Y DIRECCIONES TÉCNICAS)</v>
       </c>
-      <c r="BH3" s="96"/>
-      <c r="BI3" s="96"/>
-      <c r="BJ3" s="96"/>
-      <c r="BK3" s="96"/>
-      <c r="BL3" s="96"/>
-      <c r="BM3" s="96"/>
-      <c r="BN3" s="96"/>
-      <c r="BO3" s="96"/>
-      <c r="BP3" s="96"/>
-      <c r="BQ3" s="96"/>
-      <c r="BR3" s="96"/>
-      <c r="BS3" s="96"/>
-      <c r="BT3" s="96"/>
+      <c r="BH3" s="131"/>
+      <c r="BI3" s="131"/>
+      <c r="BJ3" s="131"/>
+      <c r="BK3" s="131"/>
+      <c r="BL3" s="131"/>
+      <c r="BM3" s="131"/>
+      <c r="BN3" s="131"/>
+      <c r="BO3" s="131"/>
+      <c r="BP3" s="131"/>
+      <c r="BQ3" s="131"/>
+      <c r="BR3" s="131"/>
+      <c r="BS3" s="131"/>
+      <c r="BT3" s="131"/>
     </row>
-    <row r="4" spans="1:72" x14ac:dyDescent="0.3">
-      <c r="A4" s="115"/>
-      <c r="B4" s="115"/>
-      <c r="C4" s="115"/>
-      <c r="D4" s="115"/>
-      <c r="E4" s="115"/>
-      <c r="F4" s="115"/>
-      <c r="G4" s="115"/>
-      <c r="H4" s="115"/>
-      <c r="I4" s="115"/>
-      <c r="J4" s="115"/>
-      <c r="K4" s="115"/>
-      <c r="L4" s="115"/>
-      <c r="M4" s="115"/>
-      <c r="N4" s="115"/>
-      <c r="O4" s="115"/>
-      <c r="P4" s="115"/>
-      <c r="Q4" s="115"/>
-      <c r="R4" s="115"/>
-      <c r="S4" s="115"/>
-      <c r="T4" s="115"/>
-      <c r="U4" s="115"/>
-      <c r="V4" s="115"/>
-      <c r="W4" s="115"/>
-      <c r="X4" s="115"/>
-      <c r="Y4" s="115"/>
-      <c r="Z4" s="115"/>
-      <c r="AA4" s="115"/>
-      <c r="AB4" s="115"/>
-      <c r="AC4" s="115"/>
-      <c r="AD4" s="115"/>
-      <c r="AE4" s="115"/>
-      <c r="AF4" s="115"/>
-      <c r="AG4" s="115"/>
-      <c r="AH4" s="115"/>
-      <c r="AI4" s="115"/>
-      <c r="AJ4" s="115"/>
-      <c r="AK4" s="115"/>
-      <c r="AL4" s="115"/>
-      <c r="AM4" s="115"/>
-      <c r="AN4" s="115"/>
-      <c r="AO4" s="115"/>
-      <c r="AP4" s="115"/>
-      <c r="AQ4" s="115"/>
-      <c r="AR4" s="115"/>
-      <c r="AS4" s="115"/>
-      <c r="AT4" s="115"/>
-      <c r="AU4" s="115"/>
-      <c r="AV4" s="115"/>
-      <c r="AW4" s="115"/>
-      <c r="AX4" s="115"/>
-      <c r="AY4" s="115"/>
-      <c r="AZ4" s="115"/>
-      <c r="BA4" s="115"/>
-      <c r="BB4" s="115"/>
-      <c r="BC4" s="115"/>
-      <c r="BD4" s="115"/>
-      <c r="BE4" s="115"/>
-      <c r="BF4" s="115"/>
-      <c r="BG4" s="95">
+    <row r="4" spans="1:72" x14ac:dyDescent="0.25">
+      <c r="A4" s="113"/>
+      <c r="B4" s="113"/>
+      <c r="C4" s="113"/>
+      <c r="D4" s="113"/>
+      <c r="E4" s="113"/>
+      <c r="F4" s="113"/>
+      <c r="G4" s="113"/>
+      <c r="H4" s="113"/>
+      <c r="I4" s="113"/>
+      <c r="J4" s="113"/>
+      <c r="K4" s="113"/>
+      <c r="L4" s="113"/>
+      <c r="M4" s="113"/>
+      <c r="N4" s="113"/>
+      <c r="O4" s="113"/>
+      <c r="P4" s="113"/>
+      <c r="Q4" s="113"/>
+      <c r="R4" s="113"/>
+      <c r="S4" s="113"/>
+      <c r="T4" s="113"/>
+      <c r="U4" s="113"/>
+      <c r="V4" s="113"/>
+      <c r="W4" s="113"/>
+      <c r="X4" s="113"/>
+      <c r="Y4" s="113"/>
+      <c r="Z4" s="113"/>
+      <c r="AA4" s="113"/>
+      <c r="AB4" s="113"/>
+      <c r="AC4" s="113"/>
+      <c r="AD4" s="113"/>
+      <c r="AE4" s="113"/>
+      <c r="AF4" s="113"/>
+      <c r="AG4" s="113"/>
+      <c r="AH4" s="113"/>
+      <c r="AI4" s="113"/>
+      <c r="AJ4" s="113"/>
+      <c r="AK4" s="113"/>
+      <c r="AL4" s="113"/>
+      <c r="AM4" s="113"/>
+      <c r="AN4" s="113"/>
+      <c r="AO4" s="113"/>
+      <c r="AP4" s="113"/>
+      <c r="AQ4" s="113"/>
+      <c r="AR4" s="113"/>
+      <c r="AS4" s="113"/>
+      <c r="AT4" s="113"/>
+      <c r="AU4" s="113"/>
+      <c r="AV4" s="113"/>
+      <c r="AW4" s="113"/>
+      <c r="AX4" s="113"/>
+      <c r="AY4" s="113"/>
+      <c r="AZ4" s="113"/>
+      <c r="BA4" s="113"/>
+      <c r="BB4" s="113"/>
+      <c r="BC4" s="113"/>
+      <c r="BD4" s="113"/>
+      <c r="BE4" s="113"/>
+      <c r="BF4" s="113"/>
+      <c r="BG4" s="130">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="BH4" s="95"/>
-      <c r="BI4" s="95"/>
-      <c r="BJ4" s="95"/>
-      <c r="BK4" s="95"/>
-      <c r="BL4" s="95"/>
-      <c r="BM4" s="95"/>
-      <c r="BN4" s="95"/>
-      <c r="BO4" s="95"/>
-      <c r="BP4" s="95"/>
-      <c r="BQ4" s="95"/>
-      <c r="BR4" s="95"/>
-      <c r="BS4" s="95"/>
-      <c r="BT4" s="95"/>
+      <c r="BH4" s="130"/>
+      <c r="BI4" s="130"/>
+      <c r="BJ4" s="130"/>
+      <c r="BK4" s="130"/>
+      <c r="BL4" s="130"/>
+      <c r="BM4" s="130"/>
+      <c r="BN4" s="130"/>
+      <c r="BO4" s="130"/>
+      <c r="BP4" s="130"/>
+      <c r="BQ4" s="130"/>
+      <c r="BR4" s="130"/>
+      <c r="BS4" s="130"/>
+      <c r="BT4" s="130"/>
     </row>
-    <row r="5" spans="1:72" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="116"/>
-      <c r="B5" s="116"/>
-      <c r="C5" s="116"/>
-      <c r="D5" s="116"/>
-      <c r="E5" s="116"/>
-      <c r="F5" s="116"/>
-      <c r="G5" s="116"/>
-      <c r="H5" s="116"/>
-      <c r="I5" s="116"/>
-      <c r="J5" s="116"/>
-      <c r="K5" s="116"/>
-      <c r="L5" s="116"/>
-      <c r="M5" s="116"/>
-      <c r="N5" s="116"/>
-      <c r="O5" s="116"/>
-      <c r="P5" s="116"/>
-      <c r="Q5" s="116"/>
-      <c r="R5" s="116"/>
-      <c r="S5" s="116"/>
-      <c r="T5" s="116"/>
-      <c r="U5" s="116"/>
-      <c r="V5" s="116"/>
-      <c r="W5" s="116"/>
-      <c r="X5" s="116"/>
-      <c r="Y5" s="116"/>
-      <c r="Z5" s="116"/>
-      <c r="AA5" s="116"/>
-      <c r="AB5" s="116"/>
-      <c r="AC5" s="116"/>
-      <c r="AD5" s="116"/>
-      <c r="AE5" s="116"/>
-      <c r="AF5" s="116"/>
-      <c r="AG5" s="116"/>
-      <c r="AH5" s="116"/>
-      <c r="AI5" s="116"/>
-      <c r="AJ5" s="116"/>
-      <c r="AK5" s="116"/>
-      <c r="AL5" s="116"/>
-      <c r="AM5" s="116"/>
-      <c r="AN5" s="116"/>
-      <c r="AO5" s="116"/>
-      <c r="AP5" s="116"/>
-      <c r="AQ5" s="116"/>
-      <c r="AR5" s="116"/>
-      <c r="AS5" s="116"/>
-      <c r="AT5" s="116"/>
-      <c r="AU5" s="116"/>
-      <c r="AV5" s="116"/>
-      <c r="AW5" s="116"/>
-      <c r="AX5" s="116"/>
-      <c r="AY5" s="116"/>
-      <c r="AZ5" s="116"/>
-      <c r="BA5" s="116"/>
-      <c r="BB5" s="116"/>
-      <c r="BC5" s="116"/>
-      <c r="BD5" s="116"/>
-      <c r="BE5" s="116"/>
-      <c r="BF5" s="116"/>
-      <c r="BG5" s="94">
+    <row r="5" spans="1:72" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="114"/>
+      <c r="B5" s="114"/>
+      <c r="C5" s="114"/>
+      <c r="D5" s="114"/>
+      <c r="E5" s="114"/>
+      <c r="F5" s="114"/>
+      <c r="G5" s="114"/>
+      <c r="H5" s="114"/>
+      <c r="I5" s="114"/>
+      <c r="J5" s="114"/>
+      <c r="K5" s="114"/>
+      <c r="L5" s="114"/>
+      <c r="M5" s="114"/>
+      <c r="N5" s="114"/>
+      <c r="O5" s="114"/>
+      <c r="P5" s="114"/>
+      <c r="Q5" s="114"/>
+      <c r="R5" s="114"/>
+      <c r="S5" s="114"/>
+      <c r="T5" s="114"/>
+      <c r="U5" s="114"/>
+      <c r="V5" s="114"/>
+      <c r="W5" s="114"/>
+      <c r="X5" s="114"/>
+      <c r="Y5" s="114"/>
+      <c r="Z5" s="114"/>
+      <c r="AA5" s="114"/>
+      <c r="AB5" s="114"/>
+      <c r="AC5" s="114"/>
+      <c r="AD5" s="114"/>
+      <c r="AE5" s="114"/>
+      <c r="AF5" s="114"/>
+      <c r="AG5" s="114"/>
+      <c r="AH5" s="114"/>
+      <c r="AI5" s="114"/>
+      <c r="AJ5" s="114"/>
+      <c r="AK5" s="114"/>
+      <c r="AL5" s="114"/>
+      <c r="AM5" s="114"/>
+      <c r="AN5" s="114"/>
+      <c r="AO5" s="114"/>
+      <c r="AP5" s="114"/>
+      <c r="AQ5" s="114"/>
+      <c r="AR5" s="114"/>
+      <c r="AS5" s="114"/>
+      <c r="AT5" s="114"/>
+      <c r="AU5" s="114"/>
+      <c r="AV5" s="114"/>
+      <c r="AW5" s="114"/>
+      <c r="AX5" s="114"/>
+      <c r="AY5" s="114"/>
+      <c r="AZ5" s="114"/>
+      <c r="BA5" s="114"/>
+      <c r="BB5" s="114"/>
+      <c r="BC5" s="114"/>
+      <c r="BD5" s="114"/>
+      <c r="BE5" s="114"/>
+      <c r="BF5" s="114"/>
+      <c r="BG5" s="129">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="BH5" s="94"/>
-      <c r="BI5" s="94"/>
-      <c r="BJ5" s="94"/>
-      <c r="BK5" s="94"/>
-      <c r="BL5" s="94"/>
-      <c r="BM5" s="94"/>
-      <c r="BN5" s="94"/>
-      <c r="BO5" s="94"/>
-      <c r="BP5" s="94"/>
-      <c r="BQ5" s="94"/>
-      <c r="BR5" s="94"/>
-      <c r="BS5" s="94"/>
-      <c r="BT5" s="94"/>
+      <c r="BH5" s="129"/>
+      <c r="BI5" s="129"/>
+      <c r="BJ5" s="129"/>
+      <c r="BK5" s="129"/>
+      <c r="BL5" s="129"/>
+      <c r="BM5" s="129"/>
+      <c r="BN5" s="129"/>
+      <c r="BO5" s="129"/>
+      <c r="BP5" s="129"/>
+      <c r="BQ5" s="129"/>
+      <c r="BR5" s="129"/>
+      <c r="BS5" s="129"/>
+      <c r="BT5" s="129"/>
     </row>
-    <row r="6" spans="1:72" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="107" t="s">
+    <row r="6" spans="1:72" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="105" t="s">
         <v>0</v>
       </c>
       <c r="B6" s="109" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="100" t="s">
+      <c r="C6" s="102" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="101"/>
-      <c r="E6" s="101"/>
-      <c r="F6" s="102"/>
-      <c r="G6" s="100" t="s">
+      <c r="D6" s="103"/>
+      <c r="E6" s="103"/>
+      <c r="F6" s="104"/>
+      <c r="G6" s="102" t="s">
         <v>20</v>
       </c>
-      <c r="H6" s="101"/>
-      <c r="I6" s="101"/>
-      <c r="J6" s="102"/>
-      <c r="K6" s="129" t="s">
+      <c r="H6" s="103"/>
+      <c r="I6" s="103"/>
+      <c r="J6" s="104"/>
+      <c r="K6" s="122" t="s">
         <v>30</v>
       </c>
-      <c r="L6" s="130"/>
-      <c r="M6" s="131"/>
-      <c r="N6" s="132"/>
-      <c r="O6" s="100" t="s">
+      <c r="L6" s="123"/>
+      <c r="M6" s="124"/>
+      <c r="N6" s="125"/>
+      <c r="O6" s="102" t="s">
         <v>19</v>
       </c>
-      <c r="P6" s="101"/>
-      <c r="Q6" s="101"/>
-      <c r="R6" s="102"/>
-      <c r="S6" s="124" t="s">
+      <c r="P6" s="103"/>
+      <c r="Q6" s="103"/>
+      <c r="R6" s="104"/>
+      <c r="S6" s="98" t="s">
         <v>2</v>
       </c>
-      <c r="T6" s="117"/>
-      <c r="U6" s="118"/>
-      <c r="V6" s="125"/>
-      <c r="W6" s="124" t="s">
+      <c r="T6" s="95"/>
+      <c r="U6" s="96"/>
+      <c r="V6" s="99"/>
+      <c r="W6" s="98" t="s">
         <v>16</v>
       </c>
-      <c r="X6" s="117"/>
-      <c r="Y6" s="118"/>
-      <c r="Z6" s="125"/>
-      <c r="AA6" s="117" t="s">
+      <c r="X6" s="95"/>
+      <c r="Y6" s="96"/>
+      <c r="Z6" s="99"/>
+      <c r="AA6" s="95" t="s">
         <v>3</v>
       </c>
-      <c r="AB6" s="117"/>
-      <c r="AC6" s="118"/>
-      <c r="AD6" s="119"/>
-      <c r="AE6" s="124" t="s">
+      <c r="AB6" s="95"/>
+      <c r="AC6" s="96"/>
+      <c r="AD6" s="97"/>
+      <c r="AE6" s="98" t="s">
         <v>26</v>
       </c>
-      <c r="AF6" s="117"/>
-      <c r="AG6" s="118"/>
-      <c r="AH6" s="125"/>
-      <c r="AI6" s="126" t="s">
+      <c r="AF6" s="95"/>
+      <c r="AG6" s="96"/>
+      <c r="AH6" s="99"/>
+      <c r="AI6" s="119" t="s">
         <v>31</v>
       </c>
-      <c r="AJ6" s="127"/>
-      <c r="AK6" s="127"/>
-      <c r="AL6" s="128"/>
-      <c r="AM6" s="124" t="s">
+      <c r="AJ6" s="120"/>
+      <c r="AK6" s="120"/>
+      <c r="AL6" s="121"/>
+      <c r="AM6" s="98" t="s">
         <v>17</v>
       </c>
-      <c r="AN6" s="117"/>
-      <c r="AO6" s="118"/>
-      <c r="AP6" s="125"/>
-      <c r="AQ6" s="124" t="s">
+      <c r="AN6" s="95"/>
+      <c r="AO6" s="96"/>
+      <c r="AP6" s="99"/>
+      <c r="AQ6" s="98" t="s">
         <v>18</v>
       </c>
-      <c r="AR6" s="117"/>
-      <c r="AS6" s="118"/>
-      <c r="AT6" s="125"/>
-      <c r="AU6" s="100" t="s">
+      <c r="AR6" s="95"/>
+      <c r="AS6" s="96"/>
+      <c r="AT6" s="99"/>
+      <c r="AU6" s="102" t="s">
         <v>21</v>
       </c>
-      <c r="AV6" s="101"/>
-      <c r="AW6" s="101"/>
-      <c r="AX6" s="102"/>
-      <c r="AY6" s="117" t="s">
+      <c r="AV6" s="103"/>
+      <c r="AW6" s="103"/>
+      <c r="AX6" s="104"/>
+      <c r="AY6" s="95" t="s">
         <v>4</v>
       </c>
-      <c r="AZ6" s="117"/>
-      <c r="BA6" s="118"/>
-      <c r="BB6" s="119"/>
-      <c r="BC6" s="120" t="s">
+      <c r="AZ6" s="95"/>
+      <c r="BA6" s="96"/>
+      <c r="BB6" s="97"/>
+      <c r="BC6" s="115" t="s">
         <v>5</v>
       </c>
-      <c r="BD6" s="121"/>
-      <c r="BE6" s="122"/>
-      <c r="BF6" s="123"/>
-      <c r="BG6" s="107" t="s">
+      <c r="BD6" s="116"/>
+      <c r="BE6" s="117"/>
+      <c r="BF6" s="118"/>
+      <c r="BG6" s="105" t="s">
         <v>0</v>
       </c>
       <c r="BH6" s="109" t="s">
         <v>1</v>
       </c>
-      <c r="BI6" s="97" t="s">
+      <c r="BI6" s="132" t="s">
         <v>15</v>
       </c>
-      <c r="BJ6" s="98"/>
-      <c r="BK6" s="98"/>
-      <c r="BL6" s="98"/>
-      <c r="BM6" s="97" t="s">
+      <c r="BJ6" s="133"/>
+      <c r="BK6" s="133"/>
+      <c r="BL6" s="133"/>
+      <c r="BM6" s="132" t="s">
         <v>8</v>
       </c>
-      <c r="BN6" s="98"/>
-      <c r="BO6" s="98"/>
-      <c r="BP6" s="99"/>
-      <c r="BQ6" s="100" t="s">
+      <c r="BN6" s="133"/>
+      <c r="BO6" s="133"/>
+      <c r="BP6" s="134"/>
+      <c r="BQ6" s="102" t="s">
         <v>20</v>
       </c>
-      <c r="BR6" s="101"/>
-      <c r="BS6" s="101"/>
-      <c r="BT6" s="102"/>
+      <c r="BR6" s="103"/>
+      <c r="BS6" s="103"/>
+      <c r="BT6" s="104"/>
     </row>
-    <row r="7" spans="1:72" x14ac:dyDescent="0.3">
-      <c r="A7" s="108"/>
+    <row r="7" spans="1:72" x14ac:dyDescent="0.25">
+      <c r="A7" s="106"/>
       <c r="B7" s="110"/>
       <c r="C7" s="2" t="s">
         <v>27</v>
@@ -2669,7 +2673,7 @@
       <c r="BF7" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="BG7" s="108"/>
+      <c r="BG7" s="106"/>
       <c r="BH7" s="110"/>
       <c r="BI7" s="11" t="s">
         <v>27</v>
@@ -2708,7 +2712,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A8" s="16">
         <v>1</v>
       </c>
@@ -2849,7 +2853,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A9" s="31">
         <v>2</v>
       </c>
@@ -2990,7 +2994,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A10" s="31">
         <v>3</v>
       </c>
@@ -3131,7 +3135,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A11" s="31">
         <v>4</v>
       </c>
@@ -3272,7 +3276,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A12" s="31">
         <v>5</v>
       </c>
@@ -3413,7 +3417,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A13" s="31">
         <v>6</v>
       </c>
@@ -3554,7 +3558,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A14" s="31">
         <v>7</v>
       </c>
@@ -3695,7 +3699,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A15" s="31">
         <v>8</v>
       </c>
@@ -3836,7 +3840,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A16" s="31">
         <v>9</v>
       </c>
@@ -3977,7 +3981,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A17" s="31">
         <v>10</v>
       </c>
@@ -4118,7 +4122,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A18" s="31">
         <v>11</v>
       </c>
@@ -4259,7 +4263,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A19" s="31">
         <v>12</v>
       </c>
@@ -4400,7 +4404,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A20" s="31">
         <v>13</v>
       </c>
@@ -4541,7 +4545,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A21" s="31">
         <v>14</v>
       </c>
@@ -4682,7 +4686,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A22" s="31">
         <v>15</v>
       </c>
@@ -4823,7 +4827,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A23" s="31">
         <v>16</v>
       </c>
@@ -4964,7 +4968,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A24" s="31">
         <v>17</v>
       </c>
@@ -5105,7 +5109,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A25" s="31">
         <v>18</v>
       </c>
@@ -5246,7 +5250,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A26" s="31">
         <v>19</v>
       </c>
@@ -5387,7 +5391,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A27" s="31">
         <v>20</v>
       </c>
@@ -5528,7 +5532,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A28" s="31">
         <v>21</v>
       </c>
@@ -5669,7 +5673,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A29" s="31">
         <v>22</v>
       </c>
@@ -5810,7 +5814,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A30" s="31">
         <v>23</v>
       </c>
@@ -5951,7 +5955,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A31" s="31">
         <v>24</v>
       </c>
@@ -6092,7 +6096,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A32" s="31">
         <v>25</v>
       </c>
@@ -6233,7 +6237,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A33" s="31">
         <v>26</v>
       </c>
@@ -6374,7 +6378,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A34" s="31">
         <v>27</v>
       </c>
@@ -6515,7 +6519,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A35" s="31">
         <v>28</v>
       </c>
@@ -6656,7 +6660,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A36" s="31">
         <v>29</v>
       </c>
@@ -6797,7 +6801,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" spans="1:72" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:72" x14ac:dyDescent="0.25">
       <c r="A37" s="47">
         <v>30</v>
       </c>
@@ -6938,11 +6942,11 @@
         <v/>
       </c>
     </row>
-    <row r="38" spans="1:72" x14ac:dyDescent="0.3">
-      <c r="A38" s="111" t="s">
+    <row r="38" spans="1:72" x14ac:dyDescent="0.25">
+      <c r="A38" s="107" t="s">
         <v>9</v>
       </c>
-      <c r="B38" s="112"/>
+      <c r="B38" s="108"/>
       <c r="C38" s="62" t="str">
         <f t="shared" ref="C38:F38" si="23">IF(SUM(C8:C37)=0,"",AVERAGE(C8:C37))</f>
         <v/>
@@ -7167,10 +7171,10 @@
         <f t="shared" si="26"/>
         <v/>
       </c>
-      <c r="BG38" s="111" t="s">
+      <c r="BG38" s="107" t="s">
         <v>9</v>
       </c>
-      <c r="BH38" s="112"/>
+      <c r="BH38" s="108"/>
       <c r="BI38" s="73" t="str">
         <f t="shared" ref="BI38:BT38" si="27">IF(SUM(BI8:BI37)=0,"",AVERAGE(BI8:BI37))</f>
         <v/>
@@ -7220,11 +7224,11 @@
         <v/>
       </c>
     </row>
-    <row r="39" spans="1:72" x14ac:dyDescent="0.3">
-      <c r="A39" s="103" t="s">
+    <row r="39" spans="1:72" x14ac:dyDescent="0.25">
+      <c r="A39" s="93" t="s">
         <v>10</v>
       </c>
-      <c r="B39" s="104"/>
+      <c r="B39" s="94"/>
       <c r="C39" s="62" t="str">
         <f t="shared" ref="C39:F39" si="28">IF(SUM(C8:C37)=0,"",MEDIAN(C8:C37))</f>
         <v/>
@@ -7449,10 +7453,10 @@
         <f t="shared" si="31"/>
         <v/>
       </c>
-      <c r="BG39" s="103" t="s">
+      <c r="BG39" s="93" t="s">
         <v>10</v>
       </c>
-      <c r="BH39" s="104"/>
+      <c r="BH39" s="94"/>
       <c r="BI39" s="73" t="str">
         <f t="shared" ref="BI39:BT39" si="32">IF(SUM(BI8:BI37)=0,"",MEDIAN(BI8:BI37))</f>
         <v/>
@@ -7502,11 +7506,11 @@
         <v/>
       </c>
     </row>
-    <row r="40" spans="1:72" x14ac:dyDescent="0.3">
-      <c r="A40" s="103" t="s">
+    <row r="40" spans="1:72" x14ac:dyDescent="0.25">
+      <c r="A40" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="B40" s="104"/>
+      <c r="B40" s="94"/>
       <c r="C40" s="62" t="str">
         <f t="shared" ref="C40:F40" si="33">IF(SUM(C8:C37)=0,"",MAX(C8:C37))</f>
         <v/>
@@ -7731,10 +7735,10 @@
         <f t="shared" si="36"/>
         <v/>
       </c>
-      <c r="BG40" s="103" t="s">
+      <c r="BG40" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="BH40" s="104"/>
+      <c r="BH40" s="94"/>
       <c r="BI40" s="73" t="str">
         <f t="shared" ref="BI40:BT40" si="37">IF(SUM(BI8:BI37)=0,"",MAX(BI8:BI37))</f>
         <v/>
@@ -7784,11 +7788,11 @@
         <v/>
       </c>
     </row>
-    <row r="41" spans="1:72" x14ac:dyDescent="0.3">
-      <c r="A41" s="103" t="s">
+    <row r="41" spans="1:72" x14ac:dyDescent="0.25">
+      <c r="A41" s="93" t="s">
         <v>12</v>
       </c>
-      <c r="B41" s="104"/>
+      <c r="B41" s="94"/>
       <c r="C41" s="62" t="str">
         <f t="shared" ref="C41:F41" si="38">IF(SUM(C8:C37)=0,"",MIN(C8:C37))</f>
         <v/>
@@ -8013,10 +8017,10 @@
         <f t="shared" si="41"/>
         <v/>
       </c>
-      <c r="BG41" s="103" t="s">
+      <c r="BG41" s="93" t="s">
         <v>12</v>
       </c>
-      <c r="BH41" s="104"/>
+      <c r="BH41" s="94"/>
       <c r="BI41" s="73" t="str">
         <f t="shared" ref="BI41:BT41" si="42">IF(SUM(BI8:BI37)=0,"",MIN(BI8:BI37))</f>
         <v/>
@@ -8066,427 +8070,433 @@
         <v/>
       </c>
     </row>
-    <row r="42" spans="1:72" x14ac:dyDescent="0.3">
-      <c r="A42" s="134" t="s">
+    <row r="42" spans="1:72" x14ac:dyDescent="0.25">
+      <c r="A42" s="100" t="s">
         <v>13</v>
       </c>
-      <c r="B42" s="135"/>
-      <c r="C42" s="77" t="str">
+      <c r="B42" s="101"/>
+      <c r="C42" s="76" t="str">
         <f t="shared" ref="C42:F42" si="43">IF(C38="","",COUNTIF(C8:C37,"&lt;51")/COUNT(C8:C37)*100)</f>
         <v/>
       </c>
-      <c r="D42" s="78" t="str">
+      <c r="D42" s="77" t="str">
         <f t="shared" ref="D42" si="44">IF(D38="","",COUNTIF(D8:D37,"&lt;51")/COUNT(D8:D37)*100)</f>
         <v/>
       </c>
-      <c r="E42" s="79" t="str">
+      <c r="E42" s="78" t="str">
         <f t="shared" si="43"/>
         <v/>
       </c>
-      <c r="F42" s="80" t="str">
+      <c r="F42" s="79" t="str">
         <f t="shared" si="43"/>
         <v/>
       </c>
-      <c r="G42" s="77" t="str">
+      <c r="G42" s="76" t="str">
         <f t="shared" ref="G42:N42" si="45">IF(G38="","",COUNTIF(G8:G37,"&lt;51")/COUNT(G8:G37)*100)</f>
         <v/>
       </c>
-      <c r="H42" s="78" t="str">
+      <c r="H42" s="77" t="str">
         <f t="shared" si="45"/>
         <v/>
       </c>
-      <c r="I42" s="79" t="str">
+      <c r="I42" s="78" t="str">
         <f t="shared" si="45"/>
         <v/>
       </c>
-      <c r="J42" s="80" t="str">
+      <c r="J42" s="79" t="str">
         <f t="shared" si="45"/>
         <v/>
       </c>
-      <c r="K42" s="77" t="str">
+      <c r="K42" s="76" t="str">
         <f t="shared" si="45"/>
         <v/>
       </c>
-      <c r="L42" s="78" t="str">
+      <c r="L42" s="77" t="str">
         <f t="shared" si="45"/>
         <v/>
       </c>
-      <c r="M42" s="79" t="str">
+      <c r="M42" s="78" t="str">
         <f t="shared" si="45"/>
         <v/>
       </c>
-      <c r="N42" s="80" t="str">
+      <c r="N42" s="79" t="str">
         <f t="shared" si="45"/>
         <v/>
       </c>
-      <c r="O42" s="78" t="str">
+      <c r="O42" s="77" t="str">
         <f t="shared" ref="O42:BF42" si="46">IF(O38="","",COUNTIF(O8:O37,"&lt;51")/COUNT(O8:O37)*100)</f>
         <v/>
       </c>
-      <c r="P42" s="78" t="str">
+      <c r="P42" s="77" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="Q42" s="79" t="str">
+      <c r="Q42" s="78" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="R42" s="81" t="str">
+      <c r="R42" s="80" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="S42" s="77" t="str">
+      <c r="S42" s="76" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="T42" s="78" t="str">
+      <c r="T42" s="77" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="U42" s="79" t="str">
+      <c r="U42" s="78" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="V42" s="80" t="str">
+      <c r="V42" s="79" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="W42" s="77" t="str">
+      <c r="W42" s="76" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="X42" s="78" t="str">
+      <c r="X42" s="77" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="Y42" s="79" t="str">
+      <c r="Y42" s="78" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="Z42" s="80" t="str">
+      <c r="Z42" s="79" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AA42" s="78" t="str">
+      <c r="AA42" s="77" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AB42" s="78" t="str">
+      <c r="AB42" s="77" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AC42" s="79" t="str">
+      <c r="AC42" s="78" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AD42" s="81" t="str">
+      <c r="AD42" s="80" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AE42" s="77" t="str">
+      <c r="AE42" s="76" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AF42" s="78" t="str">
+      <c r="AF42" s="77" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AG42" s="79" t="str">
+      <c r="AG42" s="78" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AH42" s="80" t="str">
+      <c r="AH42" s="79" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AI42" s="77" t="str">
+      <c r="AI42" s="76" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AJ42" s="78" t="str">
+      <c r="AJ42" s="77" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AK42" s="79" t="str">
+      <c r="AK42" s="78" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AL42" s="80" t="str">
+      <c r="AL42" s="79" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AM42" s="77" t="str">
+      <c r="AM42" s="76" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AN42" s="78" t="str">
+      <c r="AN42" s="77" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AO42" s="79" t="str">
+      <c r="AO42" s="78" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AP42" s="80" t="str">
+      <c r="AP42" s="79" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AQ42" s="77" t="str">
+      <c r="AQ42" s="76" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AR42" s="78" t="str">
+      <c r="AR42" s="77" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AS42" s="79" t="str">
+      <c r="AS42" s="78" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AT42" s="80" t="str">
+      <c r="AT42" s="79" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AU42" s="77" t="str">
+      <c r="AU42" s="76" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AV42" s="78" t="str">
+      <c r="AV42" s="77" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AW42" s="79" t="str">
+      <c r="AW42" s="78" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AX42" s="80" t="str">
+      <c r="AX42" s="79" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AY42" s="78" t="str">
+      <c r="AY42" s="77" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="AZ42" s="78" t="str">
+      <c r="AZ42" s="77" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="BA42" s="79" t="str">
+      <c r="BA42" s="78" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="BB42" s="81" t="str">
+      <c r="BB42" s="80" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="BC42" s="82" t="str">
+      <c r="BC42" s="81" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="BD42" s="83" t="str">
+      <c r="BD42" s="82" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="BE42" s="84" t="str">
+      <c r="BE42" s="83" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="BF42" s="85" t="str">
+      <c r="BF42" s="84" t="str">
         <f t="shared" si="46"/>
         <v/>
       </c>
-      <c r="BG42" s="105" t="s">
+      <c r="BG42" s="126" t="s">
         <v>13</v>
       </c>
-      <c r="BH42" s="106"/>
-      <c r="BI42" s="88" t="str">
+      <c r="BH42" s="127"/>
+      <c r="BI42" s="87" t="str">
         <f t="shared" ref="BI42:BT42" si="47">IF(BI38="","",COUNTIF(BI8:BI37,"&lt;51")/COUNT(BI8:BI37)*100)</f>
         <v/>
       </c>
-      <c r="BJ42" s="86" t="str">
+      <c r="BJ42" s="85" t="str">
         <f t="shared" si="47"/>
         <v/>
       </c>
-      <c r="BK42" s="87" t="str">
+      <c r="BK42" s="86" t="str">
         <f t="shared" si="47"/>
         <v/>
       </c>
-      <c r="BL42" s="89" t="str">
+      <c r="BL42" s="88" t="str">
         <f t="shared" si="47"/>
         <v/>
       </c>
-      <c r="BM42" s="88" t="str">
+      <c r="BM42" s="87" t="str">
         <f t="shared" si="47"/>
         <v/>
       </c>
-      <c r="BN42" s="86" t="str">
+      <c r="BN42" s="85" t="str">
         <f t="shared" si="47"/>
         <v/>
       </c>
-      <c r="BO42" s="87" t="str">
+      <c r="BO42" s="86" t="str">
         <f t="shared" si="47"/>
         <v/>
       </c>
-      <c r="BP42" s="89" t="str">
+      <c r="BP42" s="88" t="str">
         <f t="shared" si="47"/>
         <v/>
       </c>
-      <c r="BQ42" s="77" t="str">
+      <c r="BQ42" s="76" t="str">
         <f t="shared" si="47"/>
         <v/>
       </c>
-      <c r="BR42" s="78" t="str">
+      <c r="BR42" s="77" t="str">
         <f t="shared" si="47"/>
         <v/>
       </c>
-      <c r="BS42" s="79" t="str">
+      <c r="BS42" s="78" t="str">
         <f t="shared" si="47"/>
         <v/>
       </c>
-      <c r="BT42" s="80" t="str">
+      <c r="BT42" s="79" t="str">
         <f t="shared" si="47"/>
         <v/>
       </c>
     </row>
-    <row r="44" spans="1:72" ht="12.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="45" spans="1:72" ht="12.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="46" spans="1:72" ht="12.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="47" spans="1:72" ht="12.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="48" spans="1:72" ht="12.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="49" spans="2:77" ht="12.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="50" spans="2:77" ht="12.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="51" spans="2:77" x14ac:dyDescent="0.3">
-      <c r="B51" s="92" t="s">
+    <row r="44" spans="1:72" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="1:72" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="1:72" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="1:72" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="1:72" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="49" spans="2:82" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="50" spans="2:82" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="51" spans="2:82" x14ac:dyDescent="0.25">
+      <c r="B51" s="128" t="s">
         <v>22</v>
       </c>
-      <c r="C51" s="92"/>
-      <c r="D51" s="92"/>
-      <c r="E51" s="92"/>
-      <c r="F51" s="92"/>
-      <c r="G51" s="92"/>
-      <c r="H51" s="92"/>
-      <c r="I51" s="92"/>
-      <c r="J51" s="92"/>
+      <c r="C51" s="128"/>
+      <c r="D51" s="128"/>
+      <c r="E51" s="128"/>
+      <c r="F51" s="128"/>
+      <c r="G51" s="128"/>
+      <c r="H51" s="128"/>
+      <c r="I51" s="128"/>
+      <c r="J51" s="128"/>
       <c r="K51" s="1"/>
       <c r="L51" s="1"/>
       <c r="M51" s="1"/>
       <c r="N51" s="1"/>
       <c r="O51" s="1"/>
       <c r="P51" s="1"/>
-      <c r="Q51" s="92" t="s">
+      <c r="Q51" s="128" t="s">
         <v>22</v>
       </c>
-      <c r="R51" s="92"/>
-      <c r="S51" s="92"/>
-      <c r="T51" s="92"/>
-      <c r="U51" s="92"/>
-      <c r="V51" s="92"/>
-      <c r="W51" s="92"/>
-      <c r="X51" s="92"/>
-      <c r="Y51" s="92"/>
-      <c r="Z51" s="92"/>
-      <c r="AA51" s="92"/>
-      <c r="AB51" s="92"/>
-      <c r="AC51" s="92"/>
+      <c r="R51" s="128"/>
+      <c r="S51" s="128"/>
+      <c r="T51" s="128"/>
+      <c r="U51" s="128"/>
+      <c r="V51" s="128"/>
+      <c r="W51" s="128"/>
+      <c r="X51" s="128"/>
+      <c r="Y51" s="128"/>
+      <c r="Z51" s="128"/>
+      <c r="AA51" s="128"/>
+      <c r="AB51" s="128"/>
+      <c r="AC51" s="128"/>
       <c r="AD51" s="1"/>
       <c r="AE51" s="1"/>
       <c r="AF51" s="1"/>
       <c r="AG51" s="1"/>
-      <c r="AH51" s="92" t="s">
+      <c r="AH51" s="128" t="s">
         <v>22</v>
       </c>
-      <c r="AI51" s="92"/>
-      <c r="AJ51" s="92"/>
-      <c r="AK51" s="92"/>
-      <c r="AL51" s="92"/>
-      <c r="AM51" s="92"/>
-      <c r="AN51" s="92"/>
-      <c r="AO51" s="92"/>
-      <c r="AP51" s="92"/>
-      <c r="AQ51" s="92"/>
-      <c r="AR51" s="92"/>
-      <c r="AS51" s="92"/>
+      <c r="AI51" s="128"/>
+      <c r="AJ51" s="128"/>
+      <c r="AK51" s="128"/>
+      <c r="AL51" s="128"/>
+      <c r="AM51" s="128"/>
+      <c r="AN51" s="128"/>
+      <c r="AO51" s="128"/>
+      <c r="AP51" s="128"/>
+      <c r="AQ51" s="128"/>
+      <c r="AR51" s="128"/>
+      <c r="AS51" s="128"/>
       <c r="AT51" s="1"/>
       <c r="AU51" s="1"/>
       <c r="AV51" s="1"/>
       <c r="AW51" s="1"/>
       <c r="AX51" s="1"/>
       <c r="AY51" s="1"/>
-      <c r="BG51" s="92" t="s">
+      <c r="BG51" s="128" t="s">
         <v>22</v>
       </c>
-      <c r="BH51" s="92"/>
-      <c r="BI51" s="90"/>
-      <c r="BJ51" s="76"/>
-      <c r="BK51" s="76"/>
-      <c r="BL51" s="92" t="s">
+      <c r="BH51" s="128"/>
+      <c r="BI51" s="89"/>
+      <c r="BJ51" s="128" t="s">
         <v>22</v>
       </c>
-      <c r="BM51" s="92"/>
-      <c r="BN51" s="92"/>
-      <c r="BO51" s="92"/>
-      <c r="BP51" s="92"/>
-      <c r="BQ51" s="92"/>
-      <c r="BR51" s="92"/>
-      <c r="BS51" s="92"/>
-      <c r="BT51" s="92"/>
-      <c r="BU51" s="76"/>
-      <c r="BV51" s="76"/>
-      <c r="BW51" s="76"/>
-      <c r="BX51" s="76"/>
-      <c r="BY51" s="76"/>
+      <c r="BK51" s="128"/>
+      <c r="BL51" s="128"/>
+      <c r="BM51" s="128"/>
+      <c r="BN51" s="128"/>
+      <c r="BO51" s="128"/>
+      <c r="BP51" s="128"/>
+      <c r="BQ51" s="128"/>
+      <c r="BR51" s="128"/>
+      <c r="BS51" s="136"/>
+      <c r="BT51" s="136"/>
+      <c r="BU51" s="128" t="s">
+        <v>22</v>
+      </c>
+      <c r="BV51" s="128"/>
+      <c r="BW51" s="128"/>
+      <c r="BX51" s="128"/>
+      <c r="BY51" s="128"/>
+      <c r="BZ51" s="128"/>
+      <c r="CA51" s="128"/>
+      <c r="CB51" s="128"/>
+      <c r="CC51" s="128"/>
     </row>
-    <row r="52" spans="2:77" x14ac:dyDescent="0.3">
-      <c r="B52" s="93" t="s">
+    <row r="52" spans="2:82" x14ac:dyDescent="0.25">
+      <c r="B52" s="135" t="s">
         <v>23</v>
       </c>
-      <c r="C52" s="93"/>
-      <c r="D52" s="93"/>
-      <c r="E52" s="93"/>
-      <c r="F52" s="93"/>
-      <c r="G52" s="93"/>
-      <c r="H52" s="93"/>
-      <c r="I52" s="93"/>
-      <c r="J52" s="93"/>
+      <c r="C52" s="135"/>
+      <c r="D52" s="135"/>
+      <c r="E52" s="135"/>
+      <c r="F52" s="135"/>
+      <c r="G52" s="135"/>
+      <c r="H52" s="135"/>
+      <c r="I52" s="135"/>
+      <c r="J52" s="135"/>
       <c r="K52" s="1"/>
       <c r="L52" s="1"/>
       <c r="M52" s="1"/>
       <c r="N52" s="1"/>
       <c r="O52" s="1"/>
       <c r="P52" s="1"/>
-      <c r="Q52" s="93" t="s">
+      <c r="Q52" s="135" t="s">
         <v>24</v>
       </c>
-      <c r="R52" s="93"/>
-      <c r="S52" s="93"/>
-      <c r="T52" s="93"/>
-      <c r="U52" s="93"/>
-      <c r="V52" s="93"/>
-      <c r="W52" s="93"/>
-      <c r="X52" s="93"/>
-      <c r="Y52" s="93"/>
-      <c r="Z52" s="93"/>
-      <c r="AA52" s="93"/>
-      <c r="AB52" s="93"/>
-      <c r="AC52" s="93"/>
+      <c r="R52" s="135"/>
+      <c r="S52" s="135"/>
+      <c r="T52" s="135"/>
+      <c r="U52" s="135"/>
+      <c r="V52" s="135"/>
+      <c r="W52" s="135"/>
+      <c r="X52" s="135"/>
+      <c r="Y52" s="135"/>
+      <c r="Z52" s="135"/>
+      <c r="AA52" s="135"/>
+      <c r="AB52" s="135"/>
+      <c r="AC52" s="135"/>
       <c r="AD52" s="1"/>
       <c r="AE52" s="1"/>
       <c r="AF52" s="1"/>
       <c r="AG52" s="1"/>
-      <c r="AH52" s="93" t="s">
+      <c r="AH52" s="135" t="s">
         <v>25</v>
       </c>
-      <c r="AI52" s="93"/>
-      <c r="AJ52" s="93"/>
-      <c r="AK52" s="93"/>
-      <c r="AL52" s="93"/>
-      <c r="AM52" s="93"/>
-      <c r="AN52" s="93"/>
-      <c r="AO52" s="93"/>
-      <c r="AP52" s="93"/>
-      <c r="AQ52" s="93"/>
-      <c r="AR52" s="93"/>
-      <c r="AS52" s="93"/>
+      <c r="AI52" s="135"/>
+      <c r="AJ52" s="135"/>
+      <c r="AK52" s="135"/>
+      <c r="AL52" s="135"/>
+      <c r="AM52" s="135"/>
+      <c r="AN52" s="135"/>
+      <c r="AO52" s="135"/>
+      <c r="AP52" s="135"/>
+      <c r="AQ52" s="135"/>
+      <c r="AR52" s="135"/>
+      <c r="AS52" s="135"/>
       <c r="AT52" s="1"/>
       <c r="AU52" s="1"/>
       <c r="AV52" s="1"/>
@@ -8494,36 +8504,78 @@
       <c r="AX52" s="1"/>
       <c r="AY52" s="1"/>
       <c r="BE52" t="s">
+        <v>37</v>
+      </c>
+      <c r="BG52" s="135" t="s">
+        <v>23</v>
+      </c>
+      <c r="BH52" s="135"/>
+      <c r="BI52" s="90"/>
+      <c r="BJ52" s="135" t="s">
+        <v>24</v>
+      </c>
+      <c r="BK52" s="135"/>
+      <c r="BL52" s="135"/>
+      <c r="BM52" s="135"/>
+      <c r="BN52" s="135"/>
+      <c r="BO52" s="135"/>
+      <c r="BP52" s="135"/>
+      <c r="BQ52" s="135"/>
+      <c r="BR52" s="135"/>
+      <c r="BS52" s="75"/>
+      <c r="BT52" s="75"/>
+      <c r="BU52" s="135" t="s">
+        <v>25</v>
+      </c>
+      <c r="BV52" s="135"/>
+      <c r="BW52" s="135"/>
+      <c r="BX52" s="135"/>
+      <c r="BY52" s="135"/>
+      <c r="BZ52" s="135"/>
+      <c r="CA52" s="135"/>
+      <c r="CB52" s="135"/>
+      <c r="CC52" s="135"/>
+      <c r="CD52" s="91" t="s">
         <v>38</v>
-      </c>
-      <c r="BG52" s="93" t="s">
-        <v>23</v>
-      </c>
-      <c r="BH52" s="93"/>
-      <c r="BI52" s="91"/>
-      <c r="BJ52" s="76"/>
-      <c r="BK52" s="76"/>
-      <c r="BL52" s="93" t="s">
-        <v>25</v>
-      </c>
-      <c r="BM52" s="93"/>
-      <c r="BN52" s="93"/>
-      <c r="BO52" s="93"/>
-      <c r="BP52" s="93"/>
-      <c r="BQ52" s="93"/>
-      <c r="BR52" s="93"/>
-      <c r="BS52" s="93"/>
-      <c r="BT52" s="93"/>
-      <c r="BU52" s="76"/>
-      <c r="BV52" s="76"/>
-      <c r="BW52" s="76"/>
-      <c r="BX52" s="76"/>
-      <c r="BY52" s="75" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="49">
+  <mergeCells count="51">
+    <mergeCell ref="BU51:CC51"/>
+    <mergeCell ref="BU52:CC52"/>
+    <mergeCell ref="BJ51:BR51"/>
+    <mergeCell ref="BJ52:BR52"/>
+    <mergeCell ref="BG52:BH52"/>
+    <mergeCell ref="B51:J51"/>
+    <mergeCell ref="B52:J52"/>
+    <mergeCell ref="Q51:AC51"/>
+    <mergeCell ref="Q52:AC52"/>
+    <mergeCell ref="AH51:AS51"/>
+    <mergeCell ref="AH52:AS52"/>
+    <mergeCell ref="BG5:BT5"/>
+    <mergeCell ref="BG4:BT4"/>
+    <mergeCell ref="BG3:BT3"/>
+    <mergeCell ref="BI6:BL6"/>
+    <mergeCell ref="BM6:BP6"/>
+    <mergeCell ref="BQ6:BT6"/>
+    <mergeCell ref="BG41:BH41"/>
+    <mergeCell ref="BG42:BH42"/>
+    <mergeCell ref="BG51:BH51"/>
+    <mergeCell ref="BG6:BG7"/>
+    <mergeCell ref="BH6:BH7"/>
+    <mergeCell ref="BG38:BH38"/>
+    <mergeCell ref="BG39:BH39"/>
+    <mergeCell ref="BG40:BH40"/>
+    <mergeCell ref="A5:BF5"/>
+    <mergeCell ref="AU6:AX6"/>
+    <mergeCell ref="AY6:BB6"/>
+    <mergeCell ref="BC6:BF6"/>
+    <mergeCell ref="O6:R6"/>
+    <mergeCell ref="S6:V6"/>
+    <mergeCell ref="AI6:AL6"/>
+    <mergeCell ref="AM6:AP6"/>
+    <mergeCell ref="AQ6:AT6"/>
+    <mergeCell ref="K6:N6"/>
     <mergeCell ref="BG2:BT2"/>
     <mergeCell ref="A41:B41"/>
     <mergeCell ref="AA6:AD6"/>
@@ -8540,39 +8592,6 @@
     <mergeCell ref="A2:BF2"/>
     <mergeCell ref="A3:BF3"/>
     <mergeCell ref="A4:BF4"/>
-    <mergeCell ref="A5:BF5"/>
-    <mergeCell ref="AU6:AX6"/>
-    <mergeCell ref="AY6:BB6"/>
-    <mergeCell ref="BC6:BF6"/>
-    <mergeCell ref="O6:R6"/>
-    <mergeCell ref="S6:V6"/>
-    <mergeCell ref="AI6:AL6"/>
-    <mergeCell ref="AM6:AP6"/>
-    <mergeCell ref="AQ6:AT6"/>
-    <mergeCell ref="K6:N6"/>
-    <mergeCell ref="BG41:BH41"/>
-    <mergeCell ref="BG42:BH42"/>
-    <mergeCell ref="BG51:BH51"/>
-    <mergeCell ref="BG6:BG7"/>
-    <mergeCell ref="BH6:BH7"/>
-    <mergeCell ref="BG38:BH38"/>
-    <mergeCell ref="BG39:BH39"/>
-    <mergeCell ref="BG40:BH40"/>
-    <mergeCell ref="BG5:BT5"/>
-    <mergeCell ref="BG4:BT4"/>
-    <mergeCell ref="BG3:BT3"/>
-    <mergeCell ref="BI6:BL6"/>
-    <mergeCell ref="BM6:BP6"/>
-    <mergeCell ref="BQ6:BT6"/>
-    <mergeCell ref="BL51:BT51"/>
-    <mergeCell ref="BG52:BH52"/>
-    <mergeCell ref="BL52:BT52"/>
-    <mergeCell ref="B51:J51"/>
-    <mergeCell ref="B52:J52"/>
-    <mergeCell ref="Q51:AC51"/>
-    <mergeCell ref="Q52:AC52"/>
-    <mergeCell ref="AH51:AS51"/>
-    <mergeCell ref="AH52:AS52"/>
   </mergeCells>
   <conditionalFormatting sqref="C8:BF37 BI8:BT37">
     <cfRule type="cellIs" dxfId="1" priority="3" operator="between">

</xml_diff>